<commit_message>
Update data pasar & berita - 2026-08-25 09:56 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6525.6899</v>
+        <v>6501.667</v>
       </c>
       <c r="F2" t="n">
-        <v>24.105</v>
+        <v>-24.0229</v>
       </c>
       <c r="G2" t="n">
-        <v>0.37</v>
+        <v>-0.37</v>
       </c>
       <c r="H2" t="n">
-        <v>378269100</v>
+        <v>296534200</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>-0.28</v>
       </c>
       <c r="H3" t="n">
-        <v>2488280000</v>
+        <v>4400800000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>0.26</v>
       </c>
       <c r="H4" t="n">
-        <v>416038344</v>
+        <v>416030000</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>25980.1914</v>
+        <v>25980.1895</v>
       </c>
       <c r="F5" t="n">
-        <v>-200.2695</v>
+        <v>-200.2715</v>
       </c>
       <c r="G5" t="n">
         <v>-0.76</v>
       </c>
       <c r="H5" t="n">
-        <v>6449341000</v>
+        <v>7318150000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>66016.3594</v>
+        <v>65856.42969999999</v>
       </c>
       <c r="F6" t="n">
-        <v>-200.4297</v>
+        <v>328.3398</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.3</v>
+        <v>0.5</v>
       </c>
       <c r="H6" t="n">
-        <v>160000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>26009.4609</v>
+        <v>25511.0996</v>
       </c>
       <c r="F7" t="n">
-        <v>310.9707</v>
+        <v>-6.2305</v>
       </c>
       <c r="G7" t="n">
-        <v>1.21</v>
+        <v>-0.02</v>
       </c>
       <c r="H7" t="n">
-        <v>3350100000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3889.4448</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.4368</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.19</v>
+      </c>
       <c r="H8" t="n">
-        <v>1448500944</v>
+        <v>3462053440</v>
       </c>
     </row>
     <row r="9">
@@ -719,17 +725,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10854.3203</v>
+        <v>10861.3896</v>
       </c>
       <c r="F9" t="n">
-        <v>37.7207</v>
+        <v>7.0898</v>
       </c>
       <c r="G9" t="n">
-        <v>0.35</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>26136.5605</v>
+        <v>26285.0098</v>
       </c>
       <c r="F10" t="n">
-        <v>153.5215</v>
+        <v>178.4102</v>
       </c>
       <c r="G10" t="n">
-        <v>0.59</v>
+        <v>0.68</v>
       </c>
       <c r="H10" t="n">
-        <v>43329100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5688.96</v>
+        <v>5735.6802</v>
       </c>
       <c r="F11" t="n">
-        <v>17.0498</v>
+        <v>55.2202</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3</v>
+        <v>0.97</v>
       </c>
       <c r="H11" t="n">
-        <v>324460300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17698</v>
+        <v>17705</v>
       </c>
       <c r="F12" t="n">
-        <v>-57</v>
+        <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.32</v>
+        <v>0.28</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>98.98399999999999</v>
+        <v>98.979</v>
       </c>
       <c r="F13" t="n">
-        <v>0.184</v>
+        <v>-0.021</v>
       </c>
       <c r="G13" t="n">
-        <v>0.19</v>
+        <v>-0.02</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -889,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>159.091</v>
+        <v>159.277</v>
       </c>
       <c r="F14" t="n">
-        <v>0.208</v>
+        <v>0.373</v>
       </c>
       <c r="G14" t="n">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1038,7 +1044,7 @@
         <v>0.62</v>
       </c>
       <c r="H18" t="n">
-        <v>28999572</v>
+        <v>29015200</v>
       </c>
     </row>
     <row r="19">
@@ -1072,7 +1078,7 @@
         <v>0.11</v>
       </c>
       <c r="H19" t="n">
-        <v>20501441</v>
+        <v>20523400</v>
       </c>
     </row>
     <row r="20">
@@ -1093,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4718.7002</v>
+        <v>4694</v>
       </c>
       <c r="F20" t="n">
-        <v>94.6001</v>
+        <v>53.2002</v>
       </c>
       <c r="G20" t="n">
-        <v>2.05</v>
+        <v>1.15</v>
       </c>
       <c r="H20" t="n">
-        <v>999</v>
+        <v>75328</v>
       </c>
     </row>
     <row r="21">
@@ -1127,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>85.08</v>
+        <v>82.31</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.98</v>
+        <v>-2.7</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.27</v>
+        <v>-3.18</v>
       </c>
       <c r="H21" t="n">
-        <v>723</v>
+        <v>63605</v>
       </c>
     </row>
     <row r="22">
@@ -1161,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>92.13</v>
+        <v>87.97</v>
       </c>
       <c r="F22" t="n">
-        <v>-2.26</v>
+        <v>-4.2</v>
       </c>
       <c r="G22" t="n">
-        <v>-2.39</v>
+        <v>-4.56</v>
       </c>
       <c r="H22" t="n">
-        <v>7</v>
+        <v>10636</v>
       </c>
     </row>
     <row r="23">
@@ -1195,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.6075</v>
+        <v>6.637</v>
       </c>
       <c r="F23" t="n">
-        <v>0.028</v>
+        <v>0.038</v>
       </c>
       <c r="G23" t="n">
-        <v>0.43</v>
+        <v>0.58</v>
       </c>
       <c r="H23" t="n">
-        <v>87</v>
+        <v>10581</v>
       </c>
     </row>
     <row r="24">
@@ -1242,7 +1248,7 @@
         <v>-1.5</v>
       </c>
       <c r="H24" t="n">
-        <v>16065696</v>
+        <v>16073600</v>
       </c>
     </row>
     <row r="25">
@@ -1263,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.85</v>
+        <v>15.81</v>
       </c>
       <c r="F25" t="n">
-        <v>0.72</v>
+        <v>-0.04</v>
       </c>
       <c r="G25" t="n">
-        <v>4.76</v>
+        <v>-0.25</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1297,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>78725.63280000001</v>
+        <v>79135</v>
       </c>
       <c r="F26" t="n">
-        <v>970.3672</v>
+        <v>170.5156</v>
       </c>
       <c r="G26" t="n">
-        <v>1.25</v>
+        <v>0.22</v>
       </c>
       <c r="H26" t="n">
-        <v>55804481536</v>
+        <v>62168244224</v>
       </c>
     </row>
     <row r="27">
@@ -1743,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Genjot Produksi Emas Lewat Keterlibatan Tambang Rakyat</t>
+          <t>Puncak Kemarau, Usaha Ini Justru Diuntungkan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 22:57:44 +0700</t>
+          <t>Tue, 25 Aug 2026 16:30:31 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/02/27/berburu-emas-di-tanah-obi-10_169.jpeg?w=360&amp;amp;q=90" /&gt; Tambang rakyat akan digenjot sebagai penghasil dan pemasok emas.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/25/puncak-kemarau-usaha-ini-justru-diuntungkan-1787643855966.jpeg?w=360&amp;amp;q=90" /&gt; Puncak kemarau membawa berkah bagi pengrajin ikan asin di Muara Angke. Teriknya matahari mempercepat proses pengeringan ikan dari 3 hari menjadi ha</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8633304/genjot-produksi-emas-lewat-keterlibatan-tambang-rakyat</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8633800/puncak-kemarau-usaha-ini-justru-diuntungkan</t>
         </is>
       </c>
     </row>
@@ -1770,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KAI Poles Stasiun Cikampek, Begini Hasilnya</t>
+          <t>Prabowo Minta Menteri hingga Bos PLN Rampungkan PLTS 100 GW 3 Tahun: Bisa?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 22:46:14 +0700</t>
+          <t>Tue, 25 Aug 2026 16:20:01 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/stasiun-cikampek-1787586120884_169.jpeg?w=360&amp;amp;q=90" /&gt; Peningkatan fasilitas pelayanan di Stasiun Cikampek melalui peninggian Peron 2 dan Peron 5 serta penambahan atap overcapping.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/13/prabowo-luncurkan-motor-listrik-nasional-1786617497815_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menargetkan proyek PLTS 100 GWp selesai dalam 3 tahun. Dia meminta komitmen penuh dari jajaran menteri untuk mencapai tu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8633294/kai-poles-stasiun-cikampek-begini-hasilnya</t>
+          <t>https://finance.detik.com/energi/d-8633906/prabowo-minta-menteri-hingga-bos-pln-rampungkan-plts-100-gw-3-tahun-bisa</t>
         </is>
       </c>
     </row>
@@ -1797,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Platform Ekspor PT DSI Diluncurkan 1 September</t>
+          <t>Resmi Meluncur! 14 PLTS Ini Jadi Pembuka Megaproyek 100 GW</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 22:14:44 +0700</t>
+          <t>Tue, 25 Aug 2026 15:51:51 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496559_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Danantara Sumberdaya Indonesia (DSI) menargetkan platform tata kelola ekspor sumber daya alam (SDA) diluncurkan pada 1 September 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/25/bahlil-cek-plts-gilimanuk-1787639062029_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah Indonesia luncurkan proyek PLTS 100 GWp dengan peletakan batu pertama oleh Presiden Prabowo. Proyek ini mendukung kemandirian energi nasional.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8633276/platform-ekspor-pt-dsi-diluncurkan-1-september</t>
+          <t>https://finance.detik.com/energi/d-8633897/resmi-meluncur-14-plts-ini-jadi-pembuka-megaproyek-100-gw</t>
         </is>
       </c>
     </row>
@@ -1824,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Negosiasi Tarif Resiprokal AS Ditargetkan Rampung Tahun Ini</t>
+          <t>Megaproyek PLTS 100 GW Butuh Rp 1.140 T, Kurangi Emisi 140 Juta Ton CO2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:37:22 +0700</t>
+          <t>Tue, 25 Aug 2026 15:37:26 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/jaga-pertumbuhan-ekonomi-nasional-pemerintah-perkuat-sektor-strategis-1787215028622_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto menyebut kesepakatan tarif resiprokal Indonesia-Amerika Serikat (</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/10/solar-panel-plts-saebus-yang-berada-di-pulau-saebus-kecamatan-sapeken-kabupaten-sumenep-madura-1775792350967_169.jpeg?w=360&amp;amp;q=90" /&gt; Investasi US$ 73 miliar diperlukan untuk PLTS 100 GWp, menciptakan 5,52 juta lapangan kerja </t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633250/negosiasi-tarif-resiprokal-as-ditargetkan-rampung-tahun-ini</t>
+          <t>https://finance.detik.com/energi/d-8633876/megaproyek-plts-100-gw-butuh-rp-1-140-t-kurangi-emisi-140-juta-ton-co2</t>
         </is>
       </c>
     </row>
@@ -1851,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DSI Pantau 100 Kapal Ekspor/ Hari, Terhubung Sistem ESDM hingga Bea Cukai</t>
+          <t>Cegah Kekeringan &amp;amp; Karhutla, Langit IKN Ditebar 800 Kg Garam</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:09:35 +0700</t>
+          <t>Tue, 25 Aug 2026 15:15:42 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496617_169.jpeg?w=360&amp;amp;q=90" /&gt; Setiap hari terdapat 100 kapal melakukan pengiriman produk ke luar negeri, sehingga sulit untuk memantau aktivitas ekspor ini jika tidak ada integrasi data.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/operasi-modifikasi-cuaca-digencarkan-di-ikn-1787570076511_169.jpeg?w=360&amp;amp;q=90" /&gt; Otorita IKN bersama BMKG dan TNI AU melaksanakan Operasi Modifikasi Cuaca untuk antisipasi dampak El Nino, jaga ketersediaan air, dan mencegah </t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8633220/dsi-pantau-100-kapal-ekspor-hari-terhubung-sistem-esdm-hingga-bea-cukai</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633726/cegah-kekeringan-karhutla-langit-ikn-ditebar-800-kg-garam</t>
         </is>
       </c>
     </row>
@@ -1878,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Shana Fatina Bakal Bicara Karier Bidang Sustainability di Pertamina Talks</t>
+          <t>Pengoperasian Rute Baru LRT ke Manggarai Tunggu Peresmian Presiden</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 20:36:00 +0700</t>
+          <t>Tue, 25 Aug 2026 14:10:14 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/pertamina-1787585154509_169.png?w=360&amp;amp;q=90" /&gt; Shana Fatina, ahli energi berkelanjutan, membahas karier di bidang lingkungan dalam Pertamina Talks. Temukan bagaimana semua latar belakang bisa berkontribusi!</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/13/lrt-jakarta-fase-1b-hampir-rampung-jalur-velodrome-manggarai-segera-terhubung-1786603623025_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek LRT Jakarta Fase 1B Velodrome-Manggarai siap diresmikan besok. Panjang 12,2 km, melayani 11 stasiun, t</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633169/shana-fatina-bakal-bicara-karier-bidang-sustainability-di-pertamina-talks</t>
+          <t>https://finance.detik.com/infrastruktur/d-8633713/pengoperasian-rute-baru-lrt-ke-manggarai-tunggu-peresmian-presiden</t>
         </is>
       </c>
     </row>
@@ -1905,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PT DSI Bakal Terapkan Biaya Tata Kelola Ekspor</t>
+          <t>Saudi-Prancis Perkuat Kerja Sama Investasi, Bahas AI hingga Infrastruktur Digital</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 20:17:44 +0700</t>
+          <t>Tue, 25 Aug 2026 13:27:48 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496674_169.jpeg?w=360&amp;amp;q=90" /&gt; DSI dipastikan tidak hanya mengelola ekspor komoditas sumber daya alam (SDA) yaitu CPO, batu bara, dan ferro alloy, DSI akan menerapkan biaya ekspor.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/25/pertemuan-meja-bundar-investasi-saudi-prancis-1787639241811_169.webp?w=360&amp;amp;q=90" /&gt; Arab Saudi-Prancis perkuat hubungan ekonomi melalui pertemuan investasi di Paris. Fokus pada sektor strategis seperti AI, infrastruktur, dan </t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8633146/pt-dsi-bakal-terapkan-biaya-tata-kelola-ekspor</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633700/saudi-prancis-perkuat-kerja-sama-investasi-bahas-ai-hingga-infrastruktur-digital</t>
         </is>
       </c>
     </row>
@@ -1932,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Belajar Membatik untuk Bekal Kemandirian Ekonomi</t>
+          <t>Mimpi Prabowo Bangun PLTS 100 GW Sampai 2029, Hari Ini Baru 1,5 GW</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 20:02:43 +0700</t>
+          <t>Tue, 25 Aug 2026 13:10:05 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/belajar-membatik-untuk-bekal-kemandirian-ekonomi-1787555211021.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah warga belajar membatik di Rumah Batik Palbatu, Tebet, Jakarta Selatan, sebagai bekal keterampilan untuk membuka peluang usaha dan men</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/16/ntb-andalkan-energi-hijau-kapasitas-ebt-capai-376-mw-1760607972219_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto memulai groundbreaking PLTS 100 GWp di Bali, target rampung 2029. Proyek ini mendukung kemandirian energi da</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8632428/belajar-membatik-untuk-bekal-kemandirian-ekonomi</t>
+          <t>https://finance.detik.com/energi/d-8633667/mimpi-prabowo-bangun-plts-100-gw-sampai-2029-hari-ini-baru-1-5-gw</t>
         </is>
       </c>
     </row>
@@ -1959,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DSI Ungkap Nilai Ekspor 3 Komoditas RI Capai US$ 70 Miliar</t>
+          <t>Proyek PLTS 100 GWp Dimulai Hari Ini, Negara Bidik Hemat Rp 74 T/Tahun</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 18:37:09 +0700</t>
+          <t>Tue, 25 Aug 2026 12:25:00 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/dsi-1787569396688_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara, Rosan Roeslani, mengungkapkan nilai ekspor tiga komoditas mencapai hampir US$ 70 miliar.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/10/07/plt-hybrid-nusa-penida_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto akan meluncurkan PLTS 100 GWp pada 25 Agustus 2026 di Bali. Program ini mendukung kemandirian energi dan menciptakan lapangan kerja.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8632975/dsi-ungkap-nilai-ekspor-3-komoditas-ri-capai-us-70-miliar</t>
+          <t>https://finance.detik.com/energi/d-8633639/proyek-plts-100-gwp-dimulai-hari-ini-negara-bidik-hemat-rp-74-t-tahun</t>
         </is>
       </c>
     </row>
@@ -1986,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Susunan Lengkap Dewan Komisaris-Direksi DSI, Ada Bos Freeport</t>
+          <t>Harga Emas Hari Ini Naik Rp 18.000/Gram</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 18:23:10 +0700</t>
+          <t>Tue, 25 Aug 2026 11:12:01 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/dsi-1787569396531_43.jpeg?w=360&amp;amp;q=90" /&gt; BPI Danantara Indonesia luncurkan PT Danantara Sumber Daya Indonesia untuk memperkuat tata kelola ekspor sumber daya alam tanpa menambah birokrasi baru.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/22/harga-emas-terjun-bebas-pasar-cikini-langsung-diserbu-pembeli-1761123863235_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga emas Antam naik Rp 18.000 per gram menjadi Rp 2.768.000. Cek rincian harga emas dari 0,5 gram hingga 1.000 gram per 25 </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8632944/susunan-lengkap-dewan-komisaris-direksi-dsi-ada-bos-freeport</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633587/harga-emas-hari-ini-naik-rp-18-000-gram</t>
         </is>
       </c>
     </row>
@@ -2013,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DSI Resmi Beroperasi! Mulai Atur Ekspor Batu Bara, CPO, hingga Ferro Alloy</t>
+          <t>Jauh-Dekat Sama, Tarif LRT Manggarai ke Kelapa Gading Rp 5.000</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 18:04:19 +0700</t>
+          <t>Tue, 25 Aug 2026 10:06:14 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/dsi-1787569396616_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Danantara Sumberdaya Indonesia diluncurkan untuk tata kelola ekspor SDA yang lebih transparan dan profesional, fokus pada batu bara, CPO, dan ferro alloy.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/13/lrt-jakarta-fase-1b-hampir-rampung-jalur-velodrome-manggarai-segera-terhubung-1786603623096_169.jpeg?w=360&amp;amp;q=90" /&gt; LRT Jakarta rute Velodrome-Manggarai akan diresmikan 26 Agustus 2026 dengan tarif flat. Pembangunan rampung 1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8632919/dsi-resmi-beroperasi-mulai-atur-ekspor-batu-bara-cpo-hingga-ferro-alloy</t>
+          <t>https://finance.detik.com/infrastruktur/d-8633531/jauh-dekat-sama-tarif-lrt-manggarai-ke-kelapa-gading-rp-5-000</t>
         </is>
       </c>
     </row>
@@ -2040,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Penasihat Presiden Ungkap Buruh Jabatex Tunggu Pesangon 12 Tahun Tak Cair</t>
+          <t>PT DSI Mulai Beroperasi, Ini Susunan Pengurusnya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 18:00:47 +0700</t>
+          <t>Tue, 25 Aug 2026 09:00:04 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/14/penasihat-khusus-presiden-bidang-ketenagakerjaan-dan-kesejahteraan-buruh-said-iqbal-1784009381488_169.jpeg?w=360&amp;amp;q=90" /&gt; Pesangon sebesar Rp 59 miliar untuk sekitar 459 buruh PT Jabatex tak kunjung cair.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/dsi-1787569396531_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Danantara Sumber Daya Indonesia (DSI) resmi beroperasi.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8632901/penasihat-presiden-ungkap-buruh-jabatex-tunggu-pesangon-12-tahun-tak-cair</t>
+          <t>https://finance.detik.com/energi/d-8633419/pt-dsi-mulai-beroperasi-ini-susunan-pengurusnya</t>
         </is>
       </c>
     </row>
@@ -2067,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tok! Sarjito Terpilih Jadi Kepala Pengawas Bursa Mineral</t>
+          <t>Sambut Berkah Maulid Nabi, Mulai Langkah Finansial dengan Tabungan Emas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 18:00:20 +0700</t>
+          <t>Tue, 25 Aug 2026 08:57:12 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/calon-kepala-bursa-mineral-ojk-uji-kelayakan-di-dpr-ungkap-tantangan-industri-ri-1787560760300_169.jpeg?w=360&amp;amp;q=90" /&gt; Komisi XI DPR RI resmi menetapkan Sarjito sebagai Kepala Eksekutif Pengawas Bursa Mineral dan Komiditas St</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/25/getty-imagesreimuss-1787622988033_169.png?w=360&amp;amp;q=90" /&gt; Rayakan Maulid Nabi dengan meneladani Rasulullah dalam pengelolaan keuangan. Siapkan dana ibadah secara disiplin dengan menabung emas.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8632912/tok-sarjito-terpilih-jadi-kepala-pengawas-bursa-mineral</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633471/sambut-berkah-maulid-nabi-mulai-langkah-finansial-dengan-tabungan-emas</t>
         </is>
       </c>
     </row>
@@ -2094,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nelayan Nagekeo Belum Kembali Melaut Pascagempa</t>
+          <t>Pengusaha Akui RI Masih Dibanjiri Produk Impor Ilegal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 17:56:58 +0700</t>
+          <t>Tue, 25 Aug 2026 08:15:13 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/nelayan-nagekeo-belum-melaut-1787545775528.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah nelayan di Nagekeo, NTT, masih menambatkan perahu setelah gempa 15 Agustus 2026 karena gempa susulan dan keluarga mereka masih mengungsi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/01/25/komoditas-impor_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Apindo, Shinta Kamdani, mengungkapkan pasar Indonesia dibanjiri produk impor ilegal. Dia mendesak pemerintah untuk segera mengatasi masalah ini.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8632127/nelayan-nagekeo-belum-kembali-melaut-pascagempa</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633184/pengusaha-akui-ri-masih-dibanjiri-produk-impor-ilegal</t>
         </is>
       </c>
     </row>
@@ -2121,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IHSG Ditutup Melemah di Level 6.500</t>
+          <t>Peringatan Keras Prabowo buat Perusahaan yang Bakar Hutan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 17:43:09 +0700</t>
+          <t>Tue, 25 Aug 2026 06:45:30 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039733_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG ditutup melemah di level 6.501,66, turun 0,37%. Meskipun melemah harian, IHSG masih naik 1,56% mingguan dan 4,93% bulanan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/24/presiden-prabowo-subianto-1787553829266_169.png?w=360&amp;amp;q=90" /&gt; Peringatan keras diberikan Presiden Prabowo Subianto kepada para korporasi yang terindikasi membakar hutan.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8632888/ihsg-ditutup-melemah-di-level-6-500</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8633183/peringatan-keras-prabowo-buat-perusahaan-yang-bakar-hutan</t>
         </is>
       </c>
     </row>
@@ -2148,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ancam Pengguna Mobil Saat Penagihan, Debt Collector Ditangkap Polisi</t>
+          <t>Dukcapil Terbitkan 358 Dokumen Warga Korban Gempa di Manggarai Barat</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 25 Aug 2026 05:18:23 +0700</t>
+          <t>Tue, 25 Aug 2026 15:58:24 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Debt collector tersebut diduga melakukan pemaksaan dan penganiayaan ringan di SPBU Cengkareng.</t>
+          <t>Layanan jemput bola dan pelayanan rutin di Manggarai Barat pada hari pertama berhasil menerbitkan total 358 dokumen kependudukan.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277067/ancam-pengguna-mobil-saat-penagihan-debt-collector-ditangkap-polisi</t>
+          <t>https://www.liputan6.com/news/read/8277317/dukcapil-terbitkan-358-dokumen-warga-korban-gempa-di-manggarai-barat</t>
         </is>
       </c>
     </row>
@@ -2175,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KPI: UU Penyiaran Harus Beradaptasi dengan Era Netflix dan YouTube</t>
+          <t>Pulihkan Layanan Adminduk Pascagempa Flores, Dirjen Dukcapil Terjunkan Tim ke Ngada</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 25 Aug 2026 00:45:25 +0700</t>
+          <t>Tue, 25 Aug 2026 15:05:11 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KPI menilai revisi regulasi tersebut penting untuk menyesuaikan aturan penyiaran dengan pesatnya perkembangan teknologi.</t>
+          <t>Kemendagri memulihkan layanan administrasi kependudukan yang lumpuh dan mengganti dokumen warga yang hilang atau rusak pascagempa.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277053/kpi-uu-penyiaran-harus-beradaptasi-dengan-era-netflix-dan-youtube</t>
+          <t>https://www.liputan6.com/news/read/8277290/pulihkan-layanan-adminduk-pascagempa-flores-dirjen-dukcapil-terjunkan-tim-ke-ngada</t>
         </is>
       </c>
     </row>
@@ -2202,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kemenhut Sanksi 6 Perusahaan Buntut Kebakaran Hutan di Kalimantan</t>
+          <t>Kebakaran Hanguskan 40 Bangunan di Duren Sawit, 84 Warga Terdampak</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 23:53:17 +0700</t>
+          <t>Tue, 25 Aug 2026 15:07:37 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Total areal yang terbakar di enam perusahaan tersebut mencapai 1.511,55 hektare.</t>
+          <t>Rumah yang diduga menjadi titik awal kebakaran dalam kondisi kosong dan tidak dihuni saat kejadian.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277050/kemenhut-sanksi-6-perusahaan-buntut-kebakaran-hutan-di-kalimantan</t>
+          <t>https://www.liputan6.com/news/read/8277293/kebakaran-hanguskan-40-bangunan-di-duren-sawit-84-warga-terdampak</t>
         </is>
       </c>
     </row>
@@ -2229,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kabar Terbaru Penyidikan Kasus Korupsi MBG</t>
+          <t>LPSK: Ada Potensi Ancaman terhadap Saksi Kasus Febrie Adriansyah</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 23:42:25 +0700</t>
+          <t>Tue, 25 Aug 2026 14:49:38 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kejagung terus menggali beberapa hal dari saksi-saksi.</t>
+          <t>LPSK juga mempertimbangkan ketentuan Pasal 49 UU Nomor 3 Tahun 2026 dalam menilai permohonan FH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277048/kabar-terbaru-penyidikan-kasus-korupsi-mbg</t>
+          <t>https://www.liputan6.com/news/read/8277283/lpsk-ada-potensi-ancaman-terhadap-saksi-kasus-febrie-adriansyah</t>
         </is>
       </c>
     </row>
@@ -2256,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pesan Prabowo Saat Cek Kebakaran Hutan: Jaga Kampung Halamanmu</t>
+          <t>Gempa Magnitudo 5,1 Guncang Kepulauan Sangihe</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 23:34:06 +0700</t>
+          <t>Tue, 25 Aug 2026 13:59:49 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Prabowo meminta semua pihak untuk menjaga Jambi dan Lampung dari ancaman kebakaran hutan dan lahan.</t>
+          <t>Gempa Magnitudo 5,1 mengguncang wilayah Tahuna, Kepulauan Sangihe, Sulawesi Utara, pada Selasa (25/8/2026) pukul 13.48 WIB.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277044/pesan-prabowo-saat-cek-kebakaran-hutan-jaga-kampung-halamanmu</t>
+          <t>https://www.liputan6.com/news/read/8277264/gempa-magnitudo-51-guncang-kepulauan-sangihe</t>
         </is>
       </c>
     </row>
@@ -2283,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nasib Praperadilan Febrie Adriansyah Ditentukan Pekan Ini</t>
+          <t>Warga Terpaksa Ambil Air dari Kubangan Bekas Sawah</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 23:20:57 +0700</t>
+          <t>Tue, 25 Aug 2026 13:07:15 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kubu Febrie berharap hakim tak ragu buat keputusan.</t>
+          <t>Warga mengambil air dari kubangan bekas sawah untuk memenuhi kebutuhan sehari-hari di kawasan Weninggalih, Jonggol, Jawa Barat, Selasa, 25 Agustus 2026. Pemandangan miris ini menjadi gambaran sulitnya warga mendapatkan air bersih di tengah kekeringan. Pasokan air bersih dari Pemkab Bogor yang disalu</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277039/nasib-praperadilan-febrie-adriansyah-ditentukan-pekan-ini</t>
+          <t>https://www.liputan6.com/photo/read/8277238/warga-terpaksa-ambil-air-dari-kubangan-bekas-sawah</t>
         </is>
       </c>
     </row>
@@ -2310,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BNPB Sebut Listrik Sudah Pulih 100 Persen di NTT</t>
+          <t>Sampah Bandung Bakal Disulap Jadi Bahan Bakar</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 23:15:11 +0700</t>
+          <t>Tue, 25 Aug 2026 13:00:45 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Khusus untuk wilayah Pulau Palue, proses pemulihan layanan listrik terus dilakukan secara bertahap.</t>
+          <t>Ratusan ton sampah akan diolah menjadi bahan bakar bernilai ekonomi.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277035/bnpb-sebut-listrik-sudah-pulih-100-persen-di-ntt</t>
+          <t>https://www.liputan6.com/news/read/8276622/sampah-bandung-bakal-disulap-jadi-bahan-bakar</t>
         </is>
       </c>
     </row>
@@ -2337,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Prabowo Dorong Inovasi Baru Tangani Kebakaran Hutan, Singgung 'Ubi Bombing'</t>
+          <t>Strategi BMKG Atasi Kekeringan dan Kebakaran Hutan Kaltim</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 23:09:46 +0700</t>
+          <t>Tue, 25 Aug 2026 12:53:26 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Ubi bombing diharapkan menjadi alternatif pengganti water bombing untuk mengendalikan karhutla.</t>
+          <t>Asap kebakaran hutan juga terpantau telah melintasi wilayah Kalimantan Utara hingga Sabah, Malaysia.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277031/prabowo-dorong-inovasi-baru-tangani-kebakaran-hutan-singgung-ubi-bombing</t>
+          <t>https://www.liputan6.com/news/read/8277230/strategi-bmkg-atasi-kekeringan-dan-kebakaran-hutan-kaltim</t>
         </is>
       </c>
     </row>
@@ -2364,22 +2370,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KRL Sempat Terganggu Mobil Tertemper di Tanah Abang-Karet, Kini Kembali Normal</t>
+          <t>El Nino Perparah Kekeringan Sawah di Jonggol</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 22:47:03 +0700</t>
+          <t>Tue, 25 Aug 2026 12:30:11 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Detail kejadian belum diketahu.</t>
+          <t>Kekeringan melanda persawahan Desa Weninggalih, Kecamatan Jonggol, Kabupaten Bogor, Jawa Barat, Selasa (25/8/2026). Lahan yang retak dan mengering dimanfaatkan warga untuk menggembala ternak.
+Kondisi ini telah menyebabkan gagal panen. Pada Juli, lahan seluas 6.000 meter persegi yang biasanya mengha</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8277018/krl-sempat-terganggu-mobil-tertemper-di-tanah-abang-karet-kini-kembali-normal</t>
+          <t>https://www.liputan6.com/photo/read/8277216/el-nino-perparah-kekeringan-sawah-di-jonggol</t>
         </is>
       </c>
     </row>
@@ -2391,22 +2398,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Penggeledahan Terkait Kasus Unsoed, Dokumen Penting hingga Alat Elektronik Disita</t>
+          <t>Menag: Maulid Nabi Muhammad Momentum Jadikan Akhlak Fondasi Peradaban</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 22:02:07 +0700</t>
+          <t>Tue, 25 Aug 2026 12:36:19 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Selain rumah para tersangka, gedung rektoran juga digeledah.</t>
+          <t>Menteri Agama Nasaruddin Umar mengajak umat Islam meneladani akhlak Nabi Muhammad.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8276996/penggeledahan-terkait-kasus-unsoed-dokumen-penting-hingga-alat-elektronik-disita</t>
+          <t>https://www.liputan6.com/news/read/8277222/menag-maulid-nabi-muhammad-momentum-jadikan-akhlak-fondasi-peradaban</t>
         </is>
       </c>
     </row>
@@ -2418,22 +2425,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DPR Mulai Godok Aturan Baru Pajak Pariwisata</t>
+          <t>Prabowo Luncurkan Program PLTS 100 GW di Bali Hari Ini</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:53:33 +0700</t>
+          <t>Tue, 25 Aug 2026 10:14:45 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Baleg DPR, pemerintah, dan DPD sepakat melakukan penyesuaian Prolegnas RUU Prioritas 2026.</t>
+          <t>Program tersebut merupakan bagian dari Program Kerja Prioritas Nasional Klaster Kemandirian Energi dan Air.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8276992/dpr-mulai-godok-aturan-baru-pajak-pariwisata</t>
+          <t>https://www.liputan6.com/news/read/8277137/prabowo-luncurkan-program-plts-100-gw-di-bali-hari-ini</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2452,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jaga Jakarta Jaga Indonesia, FWJM dan Masyarakat Pandalungan Jember Kawal Stabilitas Nasional</t>
+          <t>RUU Perampasan Aset Ditargetkan Rampung Desember 2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:40:30 +0700</t>
+          <t>Tue, 25 Aug 2026 10:10:40 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FWJM dan Masyarakat Pandalungan Jember siap bertolak ke Jakarta dalam gerakan Jaga Jakarta Jaga Indonesia untuk mengawal stabilitas nasional.</t>
+          <t>Hingga saat ini, Komisi III telah menggelar 35 kali RDPU untuk menyerap aspirasi.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8276981/jaga-jakarta-jaga-indonesia-fwjm-dan-masyarakat-pandalungan-jember-kawal-stabilitas-nasional</t>
+          <t>https://www.liputan6.com/news/read/8277129/ruu-perampasan-aset-ditargetkan-rampung-desember-2026</t>
         </is>
       </c>
     </row>
@@ -2472,22 +2479,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gempa Magnitudo 6,2 Guncang Maluku Barat Daya, Tidak Berpotensi Tsunami</t>
+          <t>Kronologi Taksi Hijau Tertemper KRL Tanah Abang-Karet</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:28:06 +0700</t>
+          <t>Tue, 25 Aug 2026 09:31:57 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Titik gempa 168 km Barat Laut Maluku Barat Daya.</t>
+          <t>Akibat kejadian itu, perjalanan KA 5744B mengalami keterlambatan sekitar 30 menit</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8276980/gempa-magnitudo-62-guncang-maluku-barat-daya-tidak-berpotensi-tsunami</t>
+          <t>https://www.liputan6.com/news/read/8277117/kronologi-taksi-hijau-tertemper-krl-tanah-abang-karet</t>
         </is>
       </c>
     </row>
@@ -2499,22 +2506,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dede Yusuf Usul ASN di Tiap Kecamatan Dipangkas Jadi 15-20 Orang</t>
+          <t>Seskab Teddy: 11.567 Personel hingga 20 Ekskavator Tangani Kebakaran Hutan Sumsel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:23:56 +0700</t>
+          <t>Tue, 25 Aug 2026 08:31:00 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Saat ini jumlah ASN yang berada di kantor kecamatan bisa mencapai 40 hingga 50 orang.</t>
+          <t>Presiden Prabowo memperkuat penanganan dan pencegahan meluasnya kebakaran hutan di sejumlah provinsi.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8276978/dede-yusuf-usul-asn-di-tiap-kecamatan-dipangkas-jadi-15-20-orang</t>
+          <t>https://www.liputan6.com/news/read/8277099/seskab-teddy-11567-personel-hingga-20-ekskavator-tangani-kebakaran-hutan-sumsel</t>
         </is>
       </c>
     </row>
@@ -2526,22 +2533,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prabowo Beri Dukungan Penanganan Karhutla Kalteng dengan 3 Helikopter dan 200 Pompa Air</t>
+          <t>Kapal Induk Pertama RI Mulai Berlayar ke Indonesia</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 21:17:40 +0700</t>
+          <t>Tue, 25 Aug 2026 08:07:24 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Presiden Prabowo mengapresiasi penanganan karhutla di Kalteng dan mengerahkan 3 helikopter water bombing serta 200 pompa air.</t>
+          <t>Kapal induk Giuseppe Garibaldi akan memiliki identitas baru, KRI Gajah Mada.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8276974/prabowo-beri-dukungan-penanganan-karhutla-kalteng-dengan-3-helikopter-dan-200-pompa-air</t>
+          <t>https://www.liputan6.com/news/read/8277092/kapal-induk-pertama-ri-mulai-berlayar-ke-indonesia</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-08-30 22:01 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6521.75</v>
+        <v>6518.1211</v>
       </c>
       <c r="F2" t="n">
-        <v>116.0649</v>
+        <v>-3.6289</v>
       </c>
       <c r="G2" t="n">
-        <v>1.81</v>
+        <v>-0.06</v>
       </c>
       <c r="H2" t="n">
-        <v>282061000</v>
+        <v>266064500</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>-0.25</v>
       </c>
       <c r="H3" t="n">
-        <v>2589484000</v>
+        <v>4297560000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>-0.02</v>
       </c>
       <c r="H4" t="n">
-        <v>507511504</v>
+        <v>507510000</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26402.4238</v>
+        <v>26402.4199</v>
       </c>
       <c r="F5" t="n">
-        <v>-138.9258</v>
+        <v>-138.9297</v>
       </c>
       <c r="G5" t="n">
         <v>-0.52</v>
       </c>
       <c r="H5" t="n">
-        <v>7526280000</v>
+        <v>8457870000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>66131.97659999999</v>
+        <v>66405.5625</v>
       </c>
       <c r="F6" t="n">
-        <v>-130.1797</v>
+        <v>273.5859</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.2</v>
+        <v>0.41</v>
       </c>
       <c r="H6" t="n">
-        <v>133500000</v>
+        <v>147000000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>25565.7402</v>
+        <v>25584.7891</v>
       </c>
       <c r="F7" t="n">
-        <v>-87.23050000000001</v>
+        <v>19.0488</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.34</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>2621400000</v>
+        <v>2533500000</v>
       </c>
     </row>
     <row r="8">
@@ -694,11 +694,17 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>3952.179</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-4.3921</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.11</v>
+      </c>
       <c r="H8" t="n">
-        <v>3813524244</v>
+        <v>510600</v>
       </c>
     </row>
     <row r="9">
@@ -723,16 +729,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10824.2598</v>
+        <v>10824.2998</v>
       </c>
       <c r="F9" t="n">
-        <v>31.7598</v>
+        <v>31.7998</v>
       </c>
       <c r="G9" t="n">
         <v>0.29</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>968083200</v>
       </c>
     </row>
     <row r="10">
@@ -766,7 +772,7 @@
         <v>0.77</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>45045000</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5684.1201</v>
+        <v>5699.9302</v>
       </c>
       <c r="F11" t="n">
-        <v>-37.4697</v>
+        <v>15.8101</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.65</v>
+        <v>0.28</v>
       </c>
       <c r="H11" t="n">
-        <v>277633800</v>
+        <v>220053300</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17685</v>
+        <v>17698</v>
       </c>
       <c r="F12" t="n">
-        <v>-93</v>
+        <v>-51</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.52</v>
+        <v>-0.29</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -859,13 +865,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>99.67700000000001</v>
+        <v>99.7</v>
       </c>
       <c r="F13" t="n">
-        <v>0.517</v>
+        <v>0.54</v>
       </c>
       <c r="G13" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -889,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>160.038</v>
+        <v>160.151</v>
       </c>
       <c r="F14" t="n">
-        <v>0.783</v>
+        <v>0.83</v>
       </c>
       <c r="G14" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1038,7 +1044,7 @@
         <v>-0.3</v>
       </c>
       <c r="H18" t="n">
-        <v>35589622</v>
+        <v>35804300</v>
       </c>
     </row>
     <row r="19">
@@ -1072,7 +1078,7 @@
         <v>-0.16</v>
       </c>
       <c r="H19" t="n">
-        <v>35119569</v>
+        <v>35134500</v>
       </c>
     </row>
     <row r="20">
@@ -1097,13 +1103,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4504.1001</v>
+        <v>4529.8999</v>
       </c>
       <c r="F20" t="n">
-        <v>-105.6001</v>
+        <v>-79.80029999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>-2.29</v>
+        <v>-1.73</v>
       </c>
       <c r="H20" t="n">
         <v>268759</v>
@@ -1131,13 +1137,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>83.44</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.09</v>
+        <v>-0.13</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.11</v>
+        <v>-0.16</v>
       </c>
       <c r="H21" t="n">
         <v>142318</v>
@@ -1165,13 +1171,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>88.29000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.41</v>
+        <v>-1.6</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.57</v>
+        <v>-1.78</v>
       </c>
       <c r="H22" t="n">
         <v>25935</v>
@@ -1199,13 +1205,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.64</v>
+        <v>6.659</v>
       </c>
       <c r="F23" t="n">
-        <v>0.053</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>0.8</v>
+        <v>1.09</v>
       </c>
       <c r="H23" t="n">
         <v>37352</v>
@@ -1242,7 +1248,7 @@
         <v>-0.7</v>
       </c>
       <c r="H24" t="n">
-        <v>11717495</v>
+        <v>11763200</v>
       </c>
     </row>
     <row r="25">
@@ -1297,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>77473.99219999999</v>
+        <v>78578.1406</v>
       </c>
       <c r="F26" t="n">
-        <v>-2783.5469</v>
+        <v>747.8516</v>
       </c>
       <c r="G26" t="n">
-        <v>-3.47</v>
+        <v>0.96</v>
       </c>
       <c r="H26" t="n">
-        <v>39443300352</v>
+        <v>16119801856</v>
       </c>
     </row>
     <row r="27">
@@ -1334,9 +1340,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>1830</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-0.54</v>
+      </c>
       <c r="H27" t="n">
         <v>88806300</v>
       </c>
@@ -1362,9 +1374,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>1965</v>
+      </c>
+      <c r="F28" t="n">
+        <v>15</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.77</v>
+      </c>
       <c r="H28" t="n">
         <v>353309300</v>
       </c>
@@ -1390,9 +1408,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>810</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-0.61</v>
+      </c>
       <c r="H29" t="n">
         <v>455779700</v>
       </c>
@@ -1418,9 +1442,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>3360</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-40</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-1.18</v>
+      </c>
       <c r="H30" t="n">
         <v>18715400</v>
       </c>
@@ -1446,9 +1476,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>4990</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-85</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-1.67</v>
+      </c>
       <c r="H31" t="n">
         <v>44558500</v>
       </c>
@@ -1474,9 +1510,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>680</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
       <c r="H32" t="n">
         <v>49028400</v>
       </c>
@@ -1502,9 +1544,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>810</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-1.82</v>
+      </c>
       <c r="H33" t="n">
         <v>44065400</v>
       </c>
@@ -1530,9 +1578,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>4230</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-60</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-1.4</v>
+      </c>
       <c r="H34" t="n">
         <v>7693600</v>
       </c>
@@ -1558,9 +1612,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>725</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-1.36</v>
+      </c>
       <c r="H35" t="n">
         <v>62074100</v>
       </c>
@@ -1586,9 +1646,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>274</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-4</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-1.44</v>
+      </c>
       <c r="H36" t="n">
         <v>46464200</v>
       </c>
@@ -1614,9 +1680,15 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>9625</v>
+      </c>
+      <c r="F37" t="n">
+        <v>875</v>
+      </c>
+      <c r="G37" t="n">
+        <v>10</v>
+      </c>
       <c r="H37" t="n">
         <v>21723100</v>
       </c>
@@ -1677,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Menteri PU Percepat Pemulihan 2 Jembatan di Flores, Dibangun Lebih Tahan Gempa</t>
+          <t>GT Cipeundeuy Tol Cipali Mulai Bertarif, Ini Rinciannya</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 23:04:26 +0700</t>
+          <t>Sun, 30 Aug 2026 22:00:49 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/28/menteri-pu-cek-gempa-flores-di-manggarai-1787932879515_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pekerjaan Umum (PU) Dody Hanggodo menginstruksikan percepatan rehabilitasi Jembatan Wae Pesi di Kabupaten Manggarai dan Jembatan Wae di Ma</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/21/gerbang-tol-cipeundeuy-1787301559576_169.jpeg?w=360&amp;amp;q=90" /&gt; Gerbang Tol Cipeundeuy KM 87+950 Jalur A Tol Cikopo-Palimanan (Cipali) per hari ini mulai bertarif.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8638879/menteri-pu-percepat-pemulihan-2-jembatan-di-flores-dibangun-lebih-tahan-gempa</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640941/gt-cipeundeuy-tol-cipali-mulai-bertarif-ini-rinciannya</t>
         </is>
       </c>
     </row>
@@ -1704,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Purbaya Kasih Bocoran Insentif Dapur MBG Mau Diubah</t>
+          <t>154 Gardu Perlintasan Sebidang Dibangun buat Cegah Kecelakaan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 21:17:51 +0700</t>
+          <t>Sun, 30 Aug 2026 21:00:29 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/purbaya-1787205133556_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Purbaya Yudhi Sadewa menyampaikan rencana Badan Gizi Nasional (BGN) mengubah insentif MBG.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/30/gardu-jpl-1788092866775_169.jpeg?w=360&amp;amp;q=90" /&gt; Hingga 27 Agustus 2026, KAI Properti telah melakukan pembangunan gardu JPL pada 190 titik prioritas telah terealisasi di 154 lokasi atau mencapai 81,05%.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638791/purbaya-kasih-bocoran-insentif-dapur-mbg-mau-diubah</t>
+          <t>https://finance.detik.com/infrastruktur/d-8640936/154-gardu-perlintasan-sebidang-dibangun-buat-cegah-kecelakaan</t>
         </is>
       </c>
     </row>
@@ -1731,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MRT Jakarta Besok Buka Mulai Jam 4 Pagi, Peserta Merdeka Run Gratis</t>
+          <t>Apa Fungsi Sensus Ekonomi? Begini Penjelasan BPS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 20:27:29 +0700</t>
+          <t>Sun, 30 Aug 2026 20:00:05 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/14/perpanjangan-mrt-ke-serpong-dikebut-studi-kelayakan-dimulai-1776161234261_169.jpeg?w=360&amp;amp;q=90" /&gt; PT MRT Jakarta (Perseroda) akan menyesuaikan jam operasional layanan menjadi pukul 04.00-24.00 WIB pada Sabtu (29/8) besok.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/03/28/733b265a-ffac-48e3-88f4-32ebbd0edb20_169.jpg?w=360&amp;amp;q=90" /&gt; Sensus Ekonomi 2026 sedang dilakukan oleh Badan Pusat Statistik (BPS) sejak Mei lalu.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8638726/mrt-jakarta-besok-buka-mulai-jam-4-pagi-peserta-merdeka-run-gratis</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640782/apa-fungsi-sensus-ekonomi-begini-penjelasan-bps</t>
         </is>
       </c>
     </row>
@@ -1758,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gambir Bakal Layani Naik Turun KRL, Begini Rencana KAI</t>
+          <t>Holding Kawasan Industri Perkuat Ketahanan Sosial Masyarakat, Begini Caranya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 19:30:05 +0700</t>
+          <t>Sun, 30 Aug 2026 19:45:34 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/25/arus-balik-padati-gambir-belasan-ribu-pemudik-tiba-di-jakarta-1774437627759_169.jpeg?w=360&amp;amp;q=90" /&gt; PT KAI buka-bukaan rencana persiapan mengoperasikan Stasiun Gambir untuk sarana naik turun penumpang KRL Commuter Line.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/30/dok-danareksa-1788099318523_169.jpeg?w=360&amp;amp;q=90" /&gt; Holding Kawasan Industri memperkuat ketahanan sosial masyarakat.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8638651/gambir-bakal-layani-naik-turun-krl-begini-rencana-kai</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8641056/holding-kawasan-industri-perkuat-ketahanan-sosial-masyarakat-begini-caranya</t>
         </is>
       </c>
     </row>
@@ -1785,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bos BPS Jamin Sensus Ekonomi Bukan buat Kejar Pajak</t>
+          <t>Bank Wajib Transformasi Biar Nggak Kehilangan Nasabah</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 18:00:00 +0700</t>
+          <t>Sun, 30 Aug 2026 19:45:25 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/28/kepala-bps-1787911097039_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala BPS Amalia Adininggar Widyasanti menegaskan sensus ekonomi tidak dilakukan untuk mengejar pajak masyarakat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/12/27/ilustrasi-bank_169.png?w=360&amp;amp;q=90" /&gt; Perbankan saat ini wajib melakukan transformasi.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638544/bos-bps-jamin-sensus-ekonomi-bukan-buat-kejar-pajak</t>
+          <t>https://finance.detik.com/moneter/d-8641019/bank-wajib-transformasi-biar-nggak-kehilangan-nasabah</t>
         </is>
       </c>
     </row>
@@ -1812,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bos BPS Turun Gunung Sensus Ketua MPR Ahmad Muzani</t>
+          <t>Purbaya Buka-bukaan Rencana Ambil Alih Utang Whoosh 15 September</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 17:30:20 +0700</t>
+          <t>Sun, 30 Aug 2026 19:00:31 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/28/ketua-mpr-ahmad-muzani-melakukan-sensus-ekonomi-1787912195894_169.jpeg?w=360&amp;amp;q=90" /&gt; BPS melakukan sensus ekonomi di kediaman Ketua MPR Ahmad Muzani, mengajak masyarakat tak perlu khawatir ikut sensus.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/purbaya-1787205133714_169.jpeg?w=360&amp;amp;q=90" /&gt; Purbaya menjelaskan penyelesaian utang Whoosh ini akan melibatkan Badan Layanan Umum (BLU) atau Special Mission Vehicle (SMV) yang di bawah Kemenkeu.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638485/bos-bps-turun-gunung-sensus-ketua-mpr-ahmad-muzani</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640705/purbaya-buka-bukaan-rencana-ambil-alih-utang-whoosh-15-september</t>
         </is>
       </c>
     </row>
@@ -1839,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IHSG Terpuruk ke Zona Merah Sambut Akhir Pekan</t>
+          <t>Ekonom Sebut Tak Mudah Bikin Rupiah Menguat ke Depan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 17:28:49 +0700</t>
+          <t>Sun, 30 Aug 2026 18:00:08 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/03/ihsg-anjlok-411-persen-ke-level-5941-1780494579356_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG mengalami terpuruk ke zona hijau pada penghujung perdagangan hari ini meskipun sempat meroket sejak perdagangan dibuka.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/23/ilustrasi-uang-rupiah-1784777379320_169.jpeg?w=360&amp;amp;q=90" /&gt; Komisi XI DPR RI telah menyetujui penetapan Destry Damayanti sebagai Gubernur Bank Indonesia (BI).</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8638522/ihsg-terpuruk-ke-zona-merah-sambut-akhir-pekan</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8640775/ekonom-sebut-tak-mudah-bikin-rupiah-menguat-ke-depan</t>
         </is>
       </c>
     </row>
@@ -1866,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Viral Tukang Becak Masuk Desil 9, Bos BPS Buka Suara</t>
+          <t>Anggaran MBG &amp;amp; Pendidikan Mau Dipisah, Purbaya Kejar Pajak-Cukai yang Bocor</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:55:02 +0700</t>
+          <t>Sun, 30 Aug 2026 17:00:28 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/28/kepala-bps-1787911097039_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala BPS Amalia Widyasanti buka suara soal pengemudi becak motor yang masuk dalam desil 9 dalam data sosial ekonomi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/purbaya-1787205133643_169.jpeg?w=360&amp;amp;q=90" /&gt; Ia menjelaskan tambahan uang negara akan ditingkatkan melalui perpajakan dan cukai hasil dari menutup kebocoran yang terjadi selama ini.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638420/viral-tukang-becak-masuk-desil-9-bos-bps-buka-suara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640691/anggaran-mbg-pendidikan-mau-dipisah-purbaya-kejar-pajak-cukai-yang-bocor</t>
         </is>
       </c>
     </row>
@@ -1893,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bank SMBC Gandeng ADB Perkuat Pembiayaan Perdagangan dan Rantai Pasok</t>
+          <t>Bos BPS soal Sensus Ekonomi: Data Kami Jaga, Tak Ada Kaitannya dengan Pajak</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:42:43 +0700</t>
+          <t>Sun, 30 Aug 2026 16:00:05 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/05/adb-prospek-ekonomi-asia-ditopang-pertumbuhan-kuat-cina-dan-india_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank SMBC Indonesia Tbk menggandeng Asian Development Bank (ADB) untuk memperkuat kapabilitas pembiayaan perdagangan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/05/kepala-bps-amalia-adininggar-widyasanti-1777954089390_169.jpeg?w=360&amp;amp;q=90" /&gt; Badan Pusat Statistik (BPS) tahun ini melaksanakan Sensus Ekonomi.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638403/bank-smbc-gandeng-adb-perkuat-pembiayaan-perdagangan-dan-rantai-pasok</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640651/bos-bps-soal-sensus-ekonomi-data-kami-jaga-tak-ada-kaitannya-dengan-pajak</t>
         </is>
       </c>
     </row>
@@ -1920,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mau Wujudkan Merdeka Finansial? blu by BCA Digital Hadirkan 4 Pilar Utama</t>
+          <t>Usaha Mikro Terdampak Bencana Sumatera Bakal Dapat Bantuan Rp 3 Juta</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:38:14 +0700</t>
+          <t>Sun, 30 Aug 2026 15:30:07 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/28/mendukung-masyarakat-mewujudkan-mindset-kemerdekaan-finansial-blu-by-bca-digital-mengusung-semangat-eksplorsemaumu-1787909350469_169.jpeg?w=360&amp;amp;q=90" /&gt; blu by BCA Digital ajak masyarakat untuk mencapai kemerdekaan finansial </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/21/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1784628615964_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan anggaran senilai lebih dari Rp 1,2 triliun secara bertahap di 2026 dan 2027 untuk rehabilitasi usaha mi</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8638398/mau-wujudkan-merdeka-finansial-blu-by-bca-digital-hadirkan-4-pilar-utama</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640632/usaha-mikro-terdampak-bencana-sumatera-bakal-dapat-bantuan-rp-3-juta</t>
         </is>
       </c>
     </row>
@@ -1947,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Purbaya Gandeng Perusahaan Asing Siapkan Mesin Pendeteksi Pita Cukai Palsu</t>
+          <t>Cuma di Transmart Full Day Sale! Beli Alat Masak Jadi Semurah Ini</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:37:11 +0700</t>
+          <t>Sun, 30 Aug 2026 15:00:52 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/31/purbaya-tak-bisa-tidur-jelang-tutup-buku-apbn-2025-1767186785962_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa akan menggunakan teknologi canggih untuk memberantas peredaran pita cukai palsu.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/30/transmart-full-day-sale-1788060311914_169.png?w=360&amp;amp;q=90" /&gt; Pesta diskon Transmart Full Day Sale masih menyapa pelanggan setia seharian penuh.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638397/purbaya-gandeng-perusahaan-asing-siapkan-mesin-pendeteksi-pita-cukai-palsu</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640276/cuma-di-transmart-full-day-sale-beli-alat-masak-jadi-semurah-ini</t>
         </is>
       </c>
     </row>
@@ -1974,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Perang Dagang AS-Kanada Makin Panas, Trump Ganti Nama Danau Ontario</t>
+          <t>Yuk Miliki Hunian Impian! Ada Promo BRI Multiguna di Danantara Expo 2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:27:16 +0700</t>
+          <t>Sun, 30 Aug 2026 14:33:09 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/15/presiden-as-donald-trump-1760501717963_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Trump tandatangani perintah eksekutif ganti nama Danau Ontario jadi Danau Amerika di tengah ketegangan perang dagang dengan Kanada.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/30/magnific-1788075016778_169.jpeg?w=360&amp;amp;q=90" /&gt; Dapatkan rumah impian Anda di Danantara Housing Expo 2026! Temukan berbagai properti dan solusi pembiayaan BRI Multiguna untuk renovasi dan perabotan.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638377/perang-dagang-as-kanada-makin-panas-trump-ganti-nama-danau-ontario</t>
+          <t>https://finance.detik.com/moneter/d-8640580/yuk-miliki-hunian-impian-ada-promo-bri-multiguna-di-danantara-expo-2026</t>
         </is>
       </c>
     </row>
@@ -2001,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pertamina Siap Pimpin Pengembangan Ekosistem Carbon Capture Storage</t>
+          <t>Serbu! Tempat Tidur Diskon Gede-gedean di Transmart Full Day Sale</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:21:22 +0700</t>
+          <t>Sun, 30 Aug 2026 14:00:47 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/28/kemendagri-1787908495409_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina kembangkan ekosistem CCS/CCUS untuk mendukung Net Zero Emission 2060. Fokus pada bisnis utama dan rendah karbon, serta kolaborasi lintas industri.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/30/transmart-full-day-sale-1788060049494_169.png?w=360&amp;amp;q=90" /&gt; Gelaran diskon Transmart Full Day Sale kembali hadir menyapa pelanggan.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/ekonomi-hijau/d-8638371/pertamina-siap-pimpin-pengembangan-ekosistem-carbon-capture-storage</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640269/serbu-tempat-tidur-diskon-gede-gedean-di-transmart-full-day-sale</t>
         </is>
       </c>
     </row>
@@ -2028,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ragam Promo Kemerdekaan yang Bikin Agustusan Makin Seru, Ada Hadiah Motor!</t>
+          <t>Stasiun Gambir Bakal Dipermak Besar-besaran, Nyambung MRT-Transjakarta</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:19:32 +0700</t>
+          <t>Sun, 30 Aug 2026 13:30:27 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/02/02/ilustrasi-aplikasi-dana-1770025796767_169.png?w=360&amp;amp;q=90" /&gt; Agustus penuh promo menarik! Nikmati diskon kuliner, transportasi, belanja online, dan cicilan. Ikuti undian berhadiah Yamaha NMAX dengan DANA CICIL!</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/25/arus-balik-padati-gambir-belasan-ribu-pemudik-tiba-di-jakarta-1774437627701_169.jpeg?w=360&amp;amp;q=90" /&gt; Stasiun Gambir akan dikembangkan mengikuti kebutuhan mobilitas masyarakat yang semakin dinamis.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8638368/ragam-promo-kemerdekaan-yang-bikin-agustusan-makin-seru-ada-hadiah-motor</t>
+          <t>https://finance.detik.com/infrastruktur/d-8640498/stasiun-gambir-bakal-dipermak-besar-besaran-nyambung-mrt-transjakarta</t>
         </is>
       </c>
     </row>
@@ -2055,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pertamina Pastikan Infrastruktur Blending dan Distribusi B50 Siap</t>
+          <t>Buruh Minta RUU Perlindungan Tenaga Kerja Disahkan Oktober 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 16:17:51 +0700</t>
+          <t>Sun, 30 Aug 2026 12:37:07 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/23/b50-1784805245239_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Patra Niaga memastikan kesiapan infrastruktur blending dan distribusi B50.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/08/buruh-demo-tolak-ump-2026-minta-upah-layak-1767860482828_169.jpeg?w=360&amp;amp;q=90" /&gt; Serikat pekerja mengingatkan pemerintah soal tenggat waktu pengesahan Rancangan Undang-Undang Perlindungan Ketenagakerjaan paling lambat Oktober</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8638366/pertamina-pastikan-infrastruktur-blending-dan-distribusi-b50-siap</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8640460/buruh-minta-ruu-perlindungan-tenaga-kerja-disahkan-oktober-2026</t>
         </is>
       </c>
     </row>
@@ -2082,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Febrie Adriansyah Bantah Terima Rp 40 Miliar dari Pengusaha Tan Kian</t>
+          <t>Sosok KH Miftachul Akhyar yang Kembali Terpilih Jadi Rais Aam PBNU</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sat, 29 Aug 2026 00:34:15 +0700</t>
+          <t>Mon, 31 Aug 2026 00:12:59 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Putusan praperadilan tidak menyebut adanya kesimpulan bahwa Febrie menerima uang tersebut.</t>
+          <t>KH Miftachul Akhyar kembali terpilih menjadi Rais Aam Pengurus Besar Nahdlatul Ulama (PBNU) periode 2026-2031. Berikut profilnya.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8280058/febrie-adriansyah-bantah-terima-rp-40-miliar-dari-pengusaha-tan-kian</t>
+          <t>https://www.liputan6.com/news/read/8280915/sosok-kh-miftachul-akhyar-yang-kembali-terpilih-jadi-rais-aam-pbnu</t>
         </is>
       </c>
     </row>
@@ -2109,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Prabowo Temui Warga Relokasi Senen di Rumah Baru, Pesannya Sederhana</t>
+          <t>Muktamar ke-35 NU, KH Miftachul Akhyar Kembali Terpilih Jadi Rais Aam PBNU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sat, 29 Aug 2026 00:30:49 +0700</t>
+          <t>Sun, 30 Aug 2026 23:42:50 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mereka sebelumnya telah belasan tahun tinggal di pinggir rel kereta api kawasan Stasiun Senen, Jakarta.</t>
+          <t>Hasil musyawarah AHWA, KH Miftachul Akhyar kembali terpilih sebagai Rais Aam PBNU 2026-2031.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8280055/prabowo-temui-warga-relokasi-senen-di-rumah-baru-pesannya-sederhana</t>
+          <t>https://www.liputan6.com/news/read/8280912/muktamar-ke-35-nu-kh-miftachul-akhyar-kembali-terpilih-jadi-rais-aam-pbnu</t>
         </is>
       </c>
     </row>
@@ -2136,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Polisi Usut Dugaan Eksploitasi Anak dalam Kerusuhan Demo DPR</t>
+          <t>Bareskrim Telusuri Dugaan Perdagangan Orang Libatkan WNI di Jeju Korsel</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 23:59:45 +0700</t>
+          <t>Sun, 30 Aug 2026 22:00:21 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Penyidik menelusuri pihak yang diduga melibatkan anak-anak untuk melakukan tindakan melawan hukum dalam kerusuhan tersebut.</t>
+          <t>Nurul mengatakan informasi dugaan TPPO tersebut selanjutnya menjadi bahan pembahasan bersama.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8280047/polisi-usut-dugaan-eksploitasi-anak-dalam-kerusuhan-demo-dpr</t>
+          <t>https://www.liputan6.com/news/read/8280880/bareskrim-telusuri-dugaan-perdagangan-orang-libatkan-wni-di-jeju-korsel</t>
         </is>
       </c>
     </row>
@@ -2163,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Malam-Malam Prabowo Cek Hunian Baru Warga Bantaran Rel Senen</t>
+          <t>Gus Ipul Tanggapi Aksi Protes Massa di Muktamar ke-35 NU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 22:58:10 +0700</t>
+          <t>Sun, 30 Aug 2026 21:11:29 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Prabowo melihat langsung kondisi hunian sekaligus berinteraksi dengan warga yang kini menempati tempat tinggal baru.</t>
+          <t>Gus Ipul menyatakan keputusan terkait dinamika pencalonan Ketua Umum PBNU sepenuhnya berada di tangan peserta Muktamar.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8280029/malam-malam-prabowo-cek-hunian-baru-warga-bantaran-rel-senen</t>
+          <t>https://www.liputan6.com/news/read/8280875/gus-ipul-tanggapi-aksi-protes-massa-di-muktamar-ke-35-nu</t>
         </is>
       </c>
     </row>
@@ -2190,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alasan MK Batalkan Pasal Penghinaan Pemerintah dan DPR di KUHP</t>
+          <t>Hasil Lengkap Perolehan Suara Anggota AHWA Muktamar ke-35 NU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 22:44:41 +0700</t>
+          <t>Sun, 30 Aug 2026 20:30:21 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Menurut MK, penggunaan istilah penghinaan tersebut berpotensi menimbulkan penafsiran yang elastis dalam proses penegakan hukum.</t>
+          <t>Hasil tabulasi calon AHWA Muktamar ke-35 NU, 9 ulama raih suara tertinggi.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8280024/alasan-mk-batalkan-pasal-penghinaan-pemerintah-dan-dpr-di-kuhp</t>
+          <t>https://www.liputan6.com/news/read/8280856/hasil-lengkap-perolehan-suara-anggota-ahwa-muktamar-ke-35-nu</t>
         </is>
       </c>
     </row>
@@ -2217,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cerita Pelajar Terseret Demo Ricuh: Ditarik, Dipukul, Lalu Dipaksa Mengaku Provokator</t>
+          <t>Muktamar ke-35 NU, Ini 9 Ulama Peraih Suara Tertinggi Anggota AHWA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 22:25:06 +0700</t>
+          <t>Sun, 30 Aug 2026 20:13:29 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dia bahkan mengaku dibawa ke Polda Metro Jaya.</t>
+          <t>Berdasarkan hasil akhir, KH Nurul Huda Djazuli dari Ploso menjadi ulama dengan perolehan suara tertinggi.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8280012/cerita-pelajar-terseret-demo-ricuh-ditarik-dipukul-lalu-dipaksa-mengaku-provokator</t>
+          <t>https://www.liputan6.com/news/read/8280845/muktamar-ke-35-nu-ini-9-ulama-peraih-suara-tertinggi-anggota-ahwa</t>
         </is>
       </c>
     </row>
@@ -2244,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MK Batalkan Pasal Penghinaan Pemerintah dan Lembaga di KUHP</t>
+          <t>Update Gempa NTT: 111 Orang Meninggal, Jumlah Pengungsi Berkurang</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 21:47:08 +0700</t>
+          <t>Sun, 30 Aug 2026 18:56:21 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MK menilai ketentuan tersebut berpotensi menghilangkan hak konstitusional warga negara untuk menyampaikan pendapat.</t>
+          <t>Jumlah pengungsi per 30 Agustus 2026 pukul 07.00 WIB mencapai 188.161 orang.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279998/mk-batalkan-pasal-penghinaan-pemerintah-dan-lembaga-di-kuhp</t>
+          <t>https://www.liputan6.com/news/read/8280817/update-gempa-ntt-111-orang-meninggal-jumlah-pengungsi-berkurang</t>
         </is>
       </c>
     </row>
@@ -2271,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Polisi Duga Ada Penggerak dan Pendana Demo Rusuh Depan DPR</t>
+          <t>Aturan Jeda Politik Picu Aksi Protes di Muktamar NU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 21:22:22 +0700</t>
+          <t>Sun, 30 Aug 2026 18:45:14 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Dugaan itu muncul dalam penyidikan terhadap orang-orang yang diamankan setelah kerusuhan.</t>
+          <t>Pelaksanaan Muktamar ke-35 Nahdlatul Ulama (NU) di Pondok Pesantren Bahrul Ulum, Tambakberas, Jombang, Jawa Timur, Minggu (30/8/2026), diwarnai ketegangan. Simpatisan Gus Yusuf menggelar demonstrasi di pintu akses menuju Sidang Pleno IV. Mereka mempersoalkan aturan masa jeda satu tahun bagi mantan p</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279992/polisi-duga-ada-penggerak-dan-pendana-demo-rusuh-depan-dpr</t>
+          <t>https://www.liputan6.com/photo/read/8280813/aturan-jeda-politik-picu-aksi-protes-di-muktamar-nu</t>
         </is>
       </c>
     </row>
@@ -2298,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aturan Kepala BGN: Kepala SPPG Wajib Standby di Dapur Pukul 02.00</t>
+          <t>Kasus Kematian Bambang Masih Diselidiki, Yusril Imbau Warga Tak Terprovokasi</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 21:24:14 +0700</t>
+          <t>Sun, 30 Aug 2026 18:05:22 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kepala SPPG harus berada di dapur pada jam-jam krusial untuk memastikan seluruh standar operasional prosedur (SOP).</t>
+          <t>Menurut Yusril, penyelidikan masih dilakukan untuk mengungkap rangkaian peristiwa secara utuh dan jelas.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279993/aturan-kepala-bgn-kepala-sppg-wajib-standby-di-dapur-pukul-0200</t>
+          <t>https://www.liputan6.com/news/read/8280803/kasus-kematian-bambang-masih-diselidiki-yusril-imbau-warga-tak-terprovokasi</t>
         </is>
       </c>
     </row>
@@ -2325,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Prabowo Terima Tokoh Dayak Panglima Jilah Bahas Kebakaran Hutan Kalimantan</t>
+          <t>Putusan MK Ubah Syarat Penetapan Bencana Nasional, Ini Respons BNPB</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 21:00:01 +0700</t>
+          <t>Sun, 30 Aug 2026 17:29:11 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Panglima Jilah menyoroti tudingan terhadap masyarakat peladang sebagai penyebab kebakaran hutan Kalimantan.</t>
+          <t>BNPB buka suara soal putusan Mahkamah Konstitusi (MK) yang mengubah syarat penetapan status bencana nasional dan daerah.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279984/prabowo-terima-tokoh-dayak-panglima-jilah-bahas-kebakaran-hutan-kalimantan</t>
+          <t>https://www.liputan6.com/news/read/8280794/putusan-mk-ubah-syarat-penetapan-bencana-nasional-ini-respons-bnpb</t>
         </is>
       </c>
     </row>
@@ -2352,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Warga Tewas saat Kericuhan Pejompongan, Begini Cerita dari Keluarga</t>
+          <t>Wamendagri Minta DPRD Tingkatkan Kapasitas dan Pengawasan Pemda</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 20:41:20 +0700</t>
+          <t>Sun, 30 Aug 2026 16:41:18 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bambang sehari-hari berjualan di pinggir Jalan Pejompongan Raya.</t>
+          <t>Bima Arya soroti peran DPRD dalam menentukan dampak APBD.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279976/warga-tewas-saat-kericuhan-pejompongan-begini-cerita-dari-keluarga</t>
+          <t>https://www.liputan6.com/news/read/8280775/wamendagri-minta-dprd-tingkatkan-kapasitas-dan-pengawasan-pemda</t>
         </is>
       </c>
     </row>
@@ -2379,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Polisi Tetapkan 45 Tersangka Kerusuhan Gedung DPR</t>
+          <t>BGN Ungkap Modus Penipuan Dapur MBG</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 20:25:27 +0700</t>
+          <t>Sun, 30 Aug 2026 16:05:59 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Polisi menemukan dugaan pihak yang merekrut massa untuk kerusuhan.</t>
+          <t>BGN menegaskan tak pernah meminta uang untuk mengoperasikan dapur MBG.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279969/polisi-tetapkan-45-tersangka-kerusuhan-gedung-dpr</t>
+          <t>https://www.liputan6.com/news/read/8280759/bgn-ungkap-modus-penipuan-dapur-mbg</t>
         </is>
       </c>
     </row>
@@ -2406,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pramono Datangi Rumah Bambang, Pria Tewas saat Rusuh di Pejompongan</t>
+          <t>DPR Kawal Hak Karyawan PT Pos, Pembayaran Rp 158 Miliar Terealisasi</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 20:09:21 +0700</t>
+          <t>Sun, 30 Aug 2026 15:42:41 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pramono menemui keluarga Bambang secara tertutup sebelum melanjutkan kunjungan ke rumah Fathur, siswa yang menjadi korban pengeroyokan.</t>
+          <t>Pembayaran tagihan Rp 158 miliar memberi kepastian hak 59 ribu pekerja dan pensiunan PT Pos Indonesia.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279964/pramono-datangi-rumah-bambang-pria-tewas-saat-rusuh-di-pejompongan</t>
+          <t>https://www.liputan6.com/news/read/8280750/dpr-kawal-hak-karyawan-pt-pos-pembayaran-rp-158-miliar-terealisasi</t>
         </is>
       </c>
     </row>
@@ -2433,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Gempa Susulan di NTT Tembus 8.794 Kali</t>
+          <t>Karhutla Kalteng Belum Padam, Gubernur Agustiar Minta Sumur Bor Ditambah di Titik Rawan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 20:03:06 +0700</t>
+          <t>Sun, 30 Aug 2026 15:38:31 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Gempa susulan diperkirakan masih akan berlangsung hingga satu bulan ke depan.</t>
+          <t>Kalteng masih menghadapi 15 titik kebakaran. Gubernur Agustiar meminta sumur bor ditambah untuk mempercepat pemadaman dan pembasahan gambut.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279959/gempa-susulan-di-ntt-tembus-8794-kali</t>
+          <t>https://www.liputan6.com/news/read/8280748/karhutla-kalteng-belum-padam-gubernur-agustiar-minta-sumur-bor-ditambah-di-titik-rawan</t>
         </is>
       </c>
     </row>
@@ -2460,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Infografis: 10 Bandara Tersibuk di Dunia 2026</t>
+          <t>Kapolri Minta Garda Satya NKRI Jaga Kamtibmas</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fri, 28 Aug 2026 19:59:04 +0700</t>
+          <t>Sun, 30 Aug 2026 15:29:06 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Jutaan penumpang memadati bandara-bandara ini setiap tahun.</t>
+          <t>Kapolri mendorong Garda Satya NKRI berbuat lebih untuk bangsa.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8279946/infografis-10-bandara-tersibuk-di-dunia-2026</t>
+          <t>https://www.liputan6.com/news/read/8280741/kapolri-minta-garda-satya-nkri-jaga-kamtibmas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-09-03 22:01 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6658.1069</v>
+        <v>6595.7759</v>
       </c>
       <c r="F2" t="n">
-        <v>62.3311</v>
+        <v>-4.167</v>
       </c>
       <c r="G2" t="n">
-        <v>0.95</v>
+        <v>-0.06</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>331276500</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7666.6001</v>
+        <v>7747.71</v>
       </c>
       <c r="F3" t="n">
-        <v>35.1299</v>
+        <v>81.1099</v>
       </c>
       <c r="G3" t="n">
-        <v>0.46</v>
+        <v>1.06</v>
       </c>
       <c r="H3" t="n">
-        <v>4738910000</v>
+        <v>2695072000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>53061.9492</v>
+        <v>53686.1094</v>
       </c>
       <c r="F4" t="n">
-        <v>295.0703</v>
+        <v>624.1602</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.18</v>
       </c>
       <c r="H4" t="n">
-        <v>414520000</v>
+        <v>410262852</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26217.8301</v>
+        <v>26584.0605</v>
       </c>
       <c r="F5" t="n">
-        <v>118.0605</v>
+        <v>366.2305</v>
       </c>
       <c r="G5" t="n">
-        <v>0.45</v>
+        <v>1.4</v>
       </c>
       <c r="H5" t="n">
-        <v>7442550000</v>
+        <v>6518648000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64214.4805</v>
+        <v>64325.6406</v>
       </c>
       <c r="F6" t="n">
-        <v>-111.1602</v>
+        <v>-1889.7031</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.17</v>
+        <v>-2.85</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>172500000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>25171.0996</v>
+        <v>25311.2109</v>
       </c>
       <c r="F7" t="n">
-        <v>-140.1113</v>
+        <v>-18.5195</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.55</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2694700000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3942.0879</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.7019</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>2454378644</v>
       </c>
@@ -729,13 +723,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10750.9697</v>
+        <v>10831.5195</v>
       </c>
       <c r="F9" t="n">
-        <v>-5.5303</v>
+        <v>75.01949999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.05</v>
+        <v>0.7</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25851.1406</v>
+        <v>25839.3301</v>
       </c>
       <c r="F10" t="n">
-        <v>11.8105</v>
+        <v>-130.7793</v>
       </c>
       <c r="G10" t="n">
-        <v>0.05</v>
+        <v>-0.5</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>47864100</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5735.6802</v>
+        <v>5744.1099</v>
       </c>
       <c r="F11" t="n">
-        <v>-8.4297</v>
+        <v>33.7397</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.15</v>
+        <v>0.59</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>330116100</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17655</v>
+        <v>17684</v>
       </c>
       <c r="F12" t="n">
-        <v>-42.1992</v>
+        <v>-13.1992</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.24</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>99.242</v>
+        <v>99.003</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.318</v>
+        <v>-0.5570000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.32</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -899,13 +893,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.026</v>
+        <v>155.845</v>
       </c>
       <c r="F14" t="n">
-        <v>-3.17</v>
+        <v>-4.351</v>
       </c>
       <c r="G14" t="n">
-        <v>-1.98</v>
+        <v>-2.72</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -929,17 +923,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4796</v>
+        <v>0.4762</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>-0.0034</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>-0.71</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -963,17 +957,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5266999999999999</v>
+        <v>0.5243</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0001</v>
+        <v>-0.0024</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.02</v>
+        <v>-0.46</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -997,17 +991,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.3772</v>
+        <v>0.374</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>-0.0032</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>-0.85</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1025,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>81.95</v>
+        <v>82.06999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H18" t="n">
-        <v>21436400</v>
+        <v>18029699</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1059,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>79.11</v>
+        <v>79.20999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="G19" t="n">
-        <v>0.01</v>
+        <v>0.13</v>
       </c>
       <c r="H19" t="n">
-        <v>34409100</v>
+        <v>23037581</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1097,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4487.2998</v>
+        <v>4520.2998</v>
       </c>
       <c r="F20" t="n">
-        <v>121</v>
+        <v>154</v>
       </c>
       <c r="G20" t="n">
-        <v>2.77</v>
+        <v>3.53</v>
       </c>
       <c r="H20" t="n">
-        <v>58954</v>
+        <v>203265</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1131,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>89.88</v>
+        <v>91.67</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.13</v>
+        <v>0.66</v>
       </c>
       <c r="G21" t="n">
-        <v>-1.24</v>
+        <v>0.73</v>
       </c>
       <c r="H21" t="n">
-        <v>43058</v>
+        <v>294026</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1165,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>94.5</v>
+        <v>95.81999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.13</v>
+        <v>0.19</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.18</v>
+        <v>0.2</v>
       </c>
       <c r="H22" t="n">
-        <v>5911</v>
+        <v>47570</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1199,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.609</v>
+        <v>6.67</v>
       </c>
       <c r="F23" t="n">
-        <v>0.108</v>
+        <v>0.169</v>
       </c>
       <c r="G23" t="n">
-        <v>1.66</v>
+        <v>2.6</v>
       </c>
       <c r="H23" t="n">
-        <v>4798</v>
+        <v>31333</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1229,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>67.15000000000001</v>
+        <v>67.47</v>
       </c>
       <c r="F24" t="n">
-        <v>0.38</v>
+        <v>0.32</v>
       </c>
       <c r="G24" t="n">
-        <v>0.57</v>
+        <v>0.48</v>
       </c>
       <c r="H24" t="n">
-        <v>9798200</v>
+        <v>12193813</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1267,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.18</v>
+        <v>14.32</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.02</v>
+        <v>-0.88</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.13</v>
+        <v>-5.79</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1307,16 +1301,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>77855.02340000001</v>
+        <v>81476.63280000001</v>
       </c>
       <c r="F26" t="n">
-        <v>554.5469000000001</v>
+        <v>4176.1562</v>
       </c>
       <c r="G26" t="n">
-        <v>0.72</v>
+        <v>5.4</v>
       </c>
       <c r="H26" t="n">
-        <v>27698388992</v>
+        <v>38728830976</v>
       </c>
     </row>
     <row r="27">
@@ -1341,16 +1335,16 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1810</v>
+        <v>1800</v>
       </c>
       <c r="F27" t="n">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.55</v>
+        <v>-1.1</v>
       </c>
       <c r="H27" t="n">
-        <v>69519400</v>
+        <v>102183600</v>
       </c>
     </row>
     <row r="28">
@@ -1375,16 +1369,16 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>2030</v>
+        <v>2010</v>
       </c>
       <c r="F28" t="n">
-        <v>10</v>
+        <v>-10</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5</v>
+        <v>-0.5</v>
       </c>
       <c r="H28" t="n">
-        <v>165497700</v>
+        <v>198546700</v>
       </c>
     </row>
     <row r="29">
@@ -1418,7 +1412,7 @@
         <v>0.55</v>
       </c>
       <c r="H29" t="n">
-        <v>839642300</v>
+        <v>953565500</v>
       </c>
     </row>
     <row r="30">
@@ -1452,7 +1446,7 @@
         <v>0.3</v>
       </c>
       <c r="H30" t="n">
-        <v>16029200</v>
+        <v>18507200</v>
       </c>
     </row>
     <row r="31">
@@ -1477,16 +1471,16 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5300</v>
+        <v>5225</v>
       </c>
       <c r="F31" t="n">
-        <v>-50</v>
+        <v>-125</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.93</v>
+        <v>-2.34</v>
       </c>
       <c r="H31" t="n">
-        <v>37090300</v>
+        <v>53058300</v>
       </c>
     </row>
     <row r="32">
@@ -1511,16 +1505,16 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G32" t="n">
-        <v>0.72</v>
+        <v>1.45</v>
       </c>
       <c r="H32" t="n">
-        <v>54350100</v>
+        <v>61329400</v>
       </c>
     </row>
     <row r="33">
@@ -1554,7 +1548,7 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>68584200</v>
+        <v>76060400</v>
       </c>
     </row>
     <row r="34">
@@ -1579,16 +1573,16 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>4480</v>
+        <v>4510</v>
       </c>
       <c r="F34" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="G34" t="n">
-        <v>2.28</v>
+        <v>2.97</v>
       </c>
       <c r="H34" t="n">
-        <v>11388800</v>
+        <v>12877700</v>
       </c>
     </row>
     <row r="35">
@@ -1613,16 +1607,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="F35" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G35" t="n">
-        <v>2.6</v>
+        <v>1.95</v>
       </c>
       <c r="H35" t="n">
-        <v>112703100</v>
+        <v>124690400</v>
       </c>
     </row>
     <row r="36">
@@ -1656,7 +1650,7 @@
         <v>1.45</v>
       </c>
       <c r="H36" t="n">
-        <v>50798000</v>
+        <v>59751500</v>
       </c>
     </row>
     <row r="37">
@@ -1681,16 +1675,16 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>14550</v>
+        <v>14700</v>
       </c>
       <c r="F37" t="n">
-        <v>1800</v>
+        <v>1950</v>
       </c>
       <c r="G37" t="n">
-        <v>14.12</v>
+        <v>15.29</v>
       </c>
       <c r="H37" t="n">
-        <v>26541700</v>
+        <v>31213200</v>
       </c>
     </row>
   </sheetData>
@@ -1749,22 +1743,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Imbas Ban Pecah, Penumpang Garuda Rute Makassar-Kendari Delay 10 Jam</t>
+          <t>Utusan Khusus Presiden Bertemu Menteri PU Bahas Pembangunan Infrastruktur</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 15:13:02 +0700</t>
+          <t>Fri, 04 Sep 2026 03:37:01 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/pesawat-garuda-yang-mendarat-di-bandara-sultan-hasanuddin-makassar-mengalami-pecah-ban-1788420383765_169.jpeg?w=360&amp;amp;q=90" /&gt; Insiden ban pecah pada pesawat Garuda Indonesia menyebabkan penundaan penerbangan rute Makassar-Kend</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/04/menteri-pekerjaan-umum-pu-dody-hanggodo-menerima-kunjungan-utusan-khusus-presiden-bidang-energi-dan-iklim-hashim-djojohadikusu-1788467756524_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pekerjaan Umum (PU) Dody Hanggodo menerima kunjungan</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646822/imbas-ban-pecah-penumpang-garuda-rute-makassar-kendari-delay-10-jam</t>
+          <t>https://finance.detik.com/infrastruktur/d-8647630/utusan-khusus-presiden-bertemu-menteri-pu-bahas-pembangunan-infrastruktur</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1770,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BRI Consumer Expo 2026 Medan, Ada Bunga KPR mulai 1,75% dan KKB 1,81%</t>
+          <t>Konsultan Pajak Wajib Tahu, Sistem Coretax Bikin Cara Kerja Berubah Total</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 15:06:45 +0700</t>
+          <t>Fri, 04 Sep 2026 03:05:25 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/bri-consumer-expo-2026-medan-ada-bunga-kpr-mulai-175-dan-kkb-181-1788422716860_169.png?w=360&amp;amp;q=90" /&gt; BRI Consumer Expo 2026 Medan hadir 4-6 September, menawarkan solusi praktis untuk hunian, kendaraan, dan liburan. Temukan p</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/04/detikevent-pajak-1788465868585_169.jpeg?w=360&amp;amp;q=90" /&gt; Pelatihan &amp;amp; Sertifikasi Certified CoreTaxify Professional (CCP) Batch 7 dari Piranha Smart Center (PSC) bersama SET Academy hadir untuk profesional</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646811/bri-consumer-expo-2026-medan-ada-bunga-kpr-mulai-1-75-dan-kkb-1-81</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8647626/konsultan-pajak-wajib-tahu-sistem-coretax-bikin-cara-kerja-berubah-total</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1797,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bukan Terbitkan Surat Utang, Purbaya Sarankan Pemda Pinjam Dana dari Sini</t>
+          <t>Masih Bingung Hitung Harga Pokok Produksi? Kuasai Lewat Bootcamp Ini</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 14:37:23 +0700</t>
+          <t>Fri, 04 Sep 2026 02:42:09 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/14/menteri-keuangan-purbaya-yudhi-sadewa-1786707659025_169.png?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Purbaya Yudhi Sarewa menyarankan Pemda, termasuk Jakarta, untuk meminjam dana dari PT SMI alih-alih menerbitkan obligasi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/04/detikevent-accounting-1788464497278_169.jpeg?w=360&amp;amp;q=90" /&gt; Kelas berjalan Senin dan Selasa selama 12 kali pertemuan, mulai 14 September 2026, pukul 18.30 hingga 20.30 WIB, online lewat Zoom.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646725/bukan-terbitkan-surat-utang-purbaya-sarankan-pemda-pinjam-dana-dari-sini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8647624/masih-bingung-hitung-harga-pokok-produksi-kuasai-lewat-bootcamp-ini</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1824,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Heboh Anggaran Rp 103 M buat Podcast, Kemenkop Buka Suara</t>
+          <t>Daftar Lengkap Penerima Anugrah Ekonomi Hijau 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 14:33:35 +0700</t>
+          <t>Fri, 04 Sep 2026 02:29:30 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/sekretaris-kementerian-koperasi-sesmenkop-ahmad-zabadi-1788420644858_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Koperasi (Kemenkop) memberikan penjelasan mengenai anggaran Rp 103 miliar yang menjadi sorotan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/01/anugerah-ekonomi-hijau-1788257473437_169.jpeg?w=360&amp;amp;q=90" /&gt; Anugerah Ekonomi Hijau 2026 kembali digelar detikcom</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646717/heboh-anggaran-rp-103-m-buat-podcast-kemenkop-buka-suara</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647622/daftar-lengkap-penerima-anugrah-ekonomi-hijau-2026</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1851,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kronologi Pesawat Garuda Pecah Ban Saat Take Off dari Jakarta</t>
+          <t>Jerhemy Owen Gerakkan Anak Muda Peduli Lingkungan, Tanam Pohon hingga Kelola Sampah</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 14:10:53 +0700</t>
+          <t>Fri, 04 Sep 2026 02:25:16 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/pesawat-garuda-tujuan-makassar-alami-pecah-ban-saat-lepas-landas-dari-jakarta-1788410296815_169.jpeg?w=360&amp;amp;q=90" /&gt; Ditjen Hubud laporkan insiden pecah ban pesawat Garuda GA604. Pesawat mendarat aman di Sultan Hasanuddin, pen</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/01/anugerah-ekonomi-hijau-1788257473437_169.jpeg?w=360&amp;amp;q=90" /&gt; Kreator sekaligus aktivis lingkungan Jerhemy Owen menerima penghargaan untuk nominasi Anugerah Ekonomi Hijau.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646653/kronologi-pesawat-garuda-pecah-ban-saat-take-off-dari-jakarta</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647621/jerhemy-owen-gerakkan-anak-muda-peduli-lingkungan-tanam-pohon-hingga-kelola-sampah</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1878,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13 Bank Tutup hingga September, Begini Nasib Duit Nasabah</t>
+          <t>Dirut Jasa Raharja Raih Anugerah Ekonomi Hijau 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 14:02:34 +0700</t>
+          <t>Fri, 04 Sep 2026 02:13:34 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/10/07/gulung-tikar_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK menutup 13 BPR dan BPRS hingga September 2026. LPS jamin pengembalian dana nasabah dalam 5 hari, meski ada kendala data.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/04/anugerah-ekonomi-hijau-dirut-jasa-marga-1788462670381_169.jpeg?w=360&amp;amp;q=90" /&gt; Dirut Jasa Raharja Muhammad Awaluddin mendapat penghargaan Anugerah Ekonomi Hijau Apresiasi atas Peran Sentral Penguatan Ekosistem Keselamatan Tran</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8646636/13-bank-tutup-hingga-september-begini-nasib-duit-nasabah</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647619/dirut-jasa-raharja-raih-anugerah-ekonomi-hijau-2026</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1905,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Berburu Lowongan Kerja di Ragunan, Career Fest Jadi Harapan</t>
+          <t>Daftar Peraih Anugerah Ekonomi Hijau Kategori Komitmen Tanggung Jawab Sosial</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 14:00:01 +0700</t>
+          <t>Fri, 04 Sep 2026 01:52:48 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/berburu-lowongan-kerja-di-ragunan-career-fest-jadi-harapan-1788414921854_169.jpeg?w=360&amp;amp;q=90" /&gt; Jakarta Selatan Career Fest 2026 menyediakan 3.857 lowongan dari 37 perusahaan. Sekitar 1.000 pencari kerja telah mendaftar seca</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/01/anugerah-ekonomi-hijau-1788257473437_169.jpeg?w=360&amp;amp;q=90" /&gt; Anugerah Ekonomi Hijau kembali digelar detikcom.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8646519/berburu-lowongan-kerja-di-ragunan-career-fest-jadi-harapan</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647616/daftar-peraih-anugerah-ekonomi-hijau-kategori-komitmen-tanggung-jawab-sosial</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1932,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IPO Perusahaan Milik UGM Ditunda Gegara Belum Dapat Restu OJK</t>
+          <t>Serap 70% Tenaga Kerja Lokal, Nusantara Halmahera Minerals Dorong Pembangunan Desa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:57:06 +0700</t>
+          <t>Fri, 04 Sep 2026 00:01:11 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/02/kepala-eksekutif-pengawas-pasar-modal-keuangan-derivatif-dan-bursa-karbon-otoritas-jasa-keuangan-ojk-hasan-fawzi-1775122476252_169.jpeg?w=360&amp;amp;q=90" /&gt; Penundaan aksi korporasi perusahaan milik Universitas Gadjah Mada (UGM) in</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/anugerah-ekonomi-hijau-halmahera-minerals-1788454837220_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Nusantara Halmahera Minerals (PT NHM) memperoleh anugerah Ekonomi Hijau untuk Pemberdayaan Masyarakat dan Pengembangan Wilayah.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8646630/ipo-perusahaan-milik-ugm-ditunda-gegara-belum-dapat-restu-ojk</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647593/serap-70-tenaga-kerja-lokal-nusantara-halmahera-minerals-dorong-pembangunan-desa</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1959,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Negara Bisa Genggam Lebih dari 5% Saham Bursa</t>
+          <t>BNI Tanam 258 Ribu Mangrove, Dorong Ekonomi Pesisir Lewat Kepiting Soka-Ekowisata</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:52:44 +0700</t>
+          <t>Thu, 03 Sep 2026 23:35:23 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741182_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) buka-bukaan soal porsi saham Bursa Efek Indonesia (BEI) yang bisa digenggam oleh lembaga negara melalui me</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/anugerah-ekonomi-hijau-bni-1788453299892_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Negara Indonesia (Persero) Tbk atau BNI menerima Anugerah Ekonomi Hijau untuk Konservasi Mangrove dan Pemberdayaan Ekonomi Masyarakat Pesisir.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8646625/negara-bisa-genggam-lebih-dari-5-saham-bursa</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647582/bni-tanam-258-ribu-mangrove-dorong-ekonomi-pesisir-lewat-kepiting-soka-ekowisata</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1986,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Purbaya Pantau 5 Pegawai Pajak Paling Nakal, 3 Teratas Langsung Dirumahkan</t>
+          <t>Mitigasi Risiko Lingkungan, Triputra Agro Persada Raih Anugerah Ekonomi Hijau</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:48:36 +0700</t>
+          <t>Thu, 03 Sep 2026 23:25:02 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/menteri-keuangan-purbaya-yudhi-sadewa-1788414776895_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Purbaya Yudhi Sadewa menindak tegas pegawai pajak nakal, merumahkan 3 dari 5 pegawai teratas.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/anugerah-ekonomi-hijau-triputra-agro-1788452674428_169.jpeg?w=360&amp;amp;q=90" /&gt; Triputra Agro Persada mendapat penghargaan Anugerah Ekonomi Hijau untuk Pemberdayaan Ekonomi Masyarakat dan Mitigasi Risiko Lingkungan di Wilayah Oper</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646619/purbaya-pantau-5-pegawai-pajak-paling-nakal-3-teratas-langsung-dirumahkan</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647578/mitigasi-risiko-lingkungan-triputra-agro-persada-raih-anugerah-ekonomi-hijau</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2013,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aturan Demutualisasi Bursa Terbit Bulan Ini</t>
+          <t>BRI, Dana, hingga bank bjb Sabet Penghargaan Anugerah Ekonomi Hijau</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:33:21 +0700</t>
+          <t>Thu, 03 Sep 2026 23:15:49 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/27/kepala-eksekutif-pengawas-pasar-modal-keuangan-derivatif-dan-bursa-karbon-otoritas-jasa-keuangan-ojk-hasan-fawzi-1777264601046_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) memastikan peraturan terkait demutualisasi Bu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/01/anugerah-ekonomi-hijau-1788257473437_169.jpeg?w=360&amp;amp;q=90" /&gt; Anugerah Ekonomi Hijau 2026 resmi digelar detikcom di Menara Bank Mega, Jakarta, Kamis (3/9/2026).</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8646574/aturan-demutualisasi-bursa-terbit-bulan-ini</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647572/bri-dana-hingga-bank-bjb-sabet-penghargaan-anugerah-ekonomi-hijau</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2040,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Purbaya: Selama Saya Menteri Keuangan, Tak Ada Tax Amnesty!</t>
+          <t>Bos BGN Respons soal Siswa/Orang Tua Diminta Ambil MBG Saat Libur Karhutla</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:27:56 +0700</t>
+          <t>Thu, 03 Sep 2026 23:10:22 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/menteri-keuangan-purbaya-yudhi-sadewa-1788414776958_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Purbaya Yudhi Sadewa kembali menegaskan tidak berencana menggelar program tax amnesty atau pengampunan pajak.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/kepala-badan-gizi-nasional-sudaryono-1788451781403_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala BGN Sudaryono buka suara soal kabar siswa atau orang tua yang diminta mengambil MBG saat sekolah diliburkan akibat kebakaran hutan dan lahan (k</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646579/purbaya-selama-saya-menteri-keuangan-tak-ada-tax-amnesty</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8647570/bos-bgn-respons-soal-siswa-orang-tua-diminta-ambil-mbg-saat-libur-karhutla</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2067,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Putin Ungkap Kerja Sama Bangun Kapal-Energi Nuklir Bareng RI</t>
+          <t>Peraih Anugerah Ekonomi Hijau Pendukung Ekosistem Berkelanjutan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:22:46 +0700</t>
+          <t>Thu, 03 Sep 2026 23:00:06 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/prabowo-bertemu-putin-di-vladivostok-rusia-kamis-392029-1788415139604_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Rusia Vladimir Putin mengatakan negaranya akan mempererat kerja sama di bidang ekonomi dan perdagangan dengan Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/peraih-anugerah-ekonomi-hijau-pendukung-ekosistem-berkelanjutan-1788449531756_169.jpeg?w=360&amp;amp;q=90" /&gt; Inilah para penerima Anugerah Ekonomi Hijau Pendukung Ekosistem Berkelanjutan, di Menara Bank Mega, Jakarta, Kamis (3/9/202</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646560/putin-ungkap-kerja-sama-bangun-kapal-energi-nuklir-bareng-ri</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8647527/peraih-anugerah-ekonomi-hijau-pendukung-ekosistem-berkelanjutan</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2094,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Menanti LRT Jakarta Kelapa Gading-Manggarai Diresmikan</t>
+          <t>Daftar Perusahaan Pendukung Ekosistem Berkelanjutan Raih Anugerah Ekonomi Hijau</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:00:35 +0700</t>
+          <t>Thu, 03 Sep 2026 22:56:15 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/menanti-lrt-jakarta-kelapa-gading-manggarai-diresmikan-1788404756259_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek LRT Jakarta Kelapa Gading-Manggarai memasuki tahap akhir sebelum beroperasi penuh. Jalur sepanjang 12,2 kilometer dengan 11 s</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/01/anugerah-ekonomi-hijau-1788257473437_169.jpeg?w=360&amp;amp;q=90" /&gt; Anugerah Ekonomi Hijau 2026 resmi digelar detikcom di Menara Bank Mega, Jakarta, Kamis (3/9/2026).</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8646188/menanti-lrt-jakarta-kelapa-gading-manggarai-diresmikan</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647552/daftar-perusahaan-pendukung-ekosistem-berkelanjutan-raih-anugerah-ekonomi-hijau</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2121,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Purbaya Kasih Sinyal Pangkas Anggaran MBG Besar-besaran!</t>
+          <t>Komunikasi Berdampak, BRI Corcomm Bawa Narasi ESG Lebih Dekat ke Masyarakat</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 12:54:56 +0700</t>
+          <t>Thu, 03 Sep 2026 22:44:50 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/menteri-keuangan-purbaya-yudhi-sadewa-1788414776806_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Purbaya Yudhi Sadewa memberikan sinyal bakal memangkas anggaran program Makan Bergizi Gratis (MBG).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/anugerah-ekonomi-hijau-bri-1788450228837_169.jpeg?w=360&amp;amp;q=90" /&gt; BRI mendapatkan penghargaan Anugerah Hijau atas Komunikasi Strategis untuk Program Keberlanjutan Berdampak.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8646484/purbaya-kasih-sinyal-pangkas-anggaran-mbg-besar-besaran</t>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8647537/komunikasi-berdampak-bri-corcomm-bawa-narasi-esg-lebih-dekat-ke-masyarakat</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2148,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Isi Pertemuan 30 Menit Dedi Mulyadi dan Botok Pati Cs</t>
+          <t>Febrie Adriansyah Dicecar 50 Pertanyaan Penyidik</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 14:55:52 +0700</t>
+          <t>Thu, 03 Sep 2026 23:13:42 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pertemuan itu digelar di Lembur Pakuan, Subang, pada Selasa (1/9/2026).</t>
+          <t>Tersangka TPPU Febrie Adriansyah dicecar 50 pertanyaan selama 10 jam pemeriksaan oleh penyidik Tim 9 Kejaksaan Agung.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283812/isi-pertemuan-30-menit-dedi-mulyadi-dan-botok-pati-cs</t>
+          <t>https://www.liputan6.com/news/read/8284265/febrie-adriansyah-dicecar-50-pertanyaan-penyidik</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2175,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Putin Sambut Prabowo di Vladivostok, Singgung Hubungan Istimewa</t>
+          <t>Puluhan Kasus Keracunan Terjadi, Kepala BGN Buka Suara Soal SOP</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:46:33 +0700</t>
+          <t>Thu, 03 Sep 2026 23:00:21 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Putin mengaku senang dapat kembali bertemu dan menyambut kunjungan Prabowo di Rusia.</t>
+          <t>BGN mengungkapkan 80–90 persen kasus keracunan program Makan Bergizi Gratis dipicu pelanggaran SOP waktu penyajian dan kapasitas dapur.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283781/putin-sambut-prabowo-di-vladivostok-singgung-hubungan-istimewa</t>
+          <t>https://www.liputan6.com/news/read/8284260/puluhan-kasus-keracunan-terjadi-kepala-bgn-buka-suara-soal-sop</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2202,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tips Cegah Kebakaran Saat Musim Kemarau dari Damkar</t>
+          <t>Kemendagri Dorong Mahasiswa Jadi Garda Terdepan Penanganan TBC di Tingkat Desa</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:40:12 +0700</t>
+          <t>Thu, 03 Sep 2026 22:43:24 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Dinas Penanggulangan Kebakaran dan Penyelamatan DKI Jakarta membagikan sejumlah langkah mencegah kebakaran.</t>
+          <t>Kemendagri mendorong mobilisasi mahasiswa ke tingkat desa guna memperkuat penanganan dan eliminasi TBC nasional.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283774/tips-cegah-kebakaran-saat-musim-kemarau-dari-damkar</t>
+          <t>https://www.liputan6.com/news/read/8284257/kemendagri-dorong-mahasiswa-jadi-garda-terdepan-penanganan-tbc-di-tingkat-desa</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2229,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bandar Obat Keras Tanah Abang Ditangkap</t>
+          <t>Banyak Pemotor Lawan Arus, Pembatas Jalan Yos Sudarso Jakut Diperpanjang</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:10:00 +0700</t>
+          <t>Thu, 03 Sep 2026 22:33:42 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Penangkapan ini lanjutan dari pengungkapan kasus peredaran obat ilegal dengan barang bukti fantastis.</t>
+          <t>Langkah penambahan pembatas jalan diambil akibat maraknya pengendara sepeda motor yang nekat melawan arus demi menerobos jalur.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283752/bandar-obat-keras-tanah-abang-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8284256/banyak-pemotor-lawan-arus-pembatas-jalan-yos-sudarso-jakut-diperpanjang</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2256,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Putin dan Prabowo Bahas Kerja Sama Kapal hingga Nuklir</t>
+          <t>Skema Baru Insentif SPPG: Tak Lagi Rata Rp 6 Juta per Hari</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:04:24 +0700</t>
+          <t>Thu, 03 Sep 2026 21:56:24 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Putin menyebut hubungan Indonesia-Rusia berpotensi terus berkembang.</t>
+          <t>Badan Gizi Nasional (BGN) tengah menyiapkan perubahan skema insentif, besaran intensif tidak lagi dipukul rata Rp 6 juta per hari untuk setiap dapur.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283747/putin-dan-prabowo-bahas-kerja-sama-kapal-hingga-nuklir</t>
+          <t>https://www.liputan6.com/news/read/8284244/skema-baru-insentif-sppg-tak-lagi-rata-rp-6-juta-per-hari</t>
         </is>
       </c>
     </row>
@@ -2289,23 +2283,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Eks Jampidsus Febrie Adriansyah Kembali Diperiksa Kejagung</t>
+          <t>Kejagung Dalami Dugaan Aliran Dana Rp 40 Miliar dari Tan Kian</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:00:53 +0700</t>
+          <t>Thu, 03 Sep 2026 21:41:31 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kejaksaan Agung menjadwalkan pemeriksaan eks Jampidsus Febrie Adriansyah pada Kamis, 3 September 2026. Febrie diperiksa sebagai saksi dalam perkara dugaan tindak pidana pencucian uang (TPPU).
-Sebelumnya, Febrie diperiksa tim sembilan Kejagung pada 7 Agustus 2026 sebagai tersangka sekaligus saksi. I</t>
+          <t>Kejagung menyebut dugaan aliran dana yang muncul dalam sidang praperadilan Febrie Adriansyah masih didalami dan akan diuji dalam pokok perkara.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/photo/read/8283741/eks-jampidsus-febrie-adriansyah-kembali-diperiksa-kejagung</t>
+          <t>https://www.liputan6.com/news/read/8284238/kejagung-dalami-dugaan-aliran-dana-rp-40-miliar-dari-tan-kian</t>
         </is>
       </c>
     </row>
@@ -2317,22 +2310,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pria Nekat Curi Laptop dan iPhone di Mal, Lalu Disembunyikan Dalam Celana</t>
+          <t>BGN Batalkan Pengadaan LED Rp535 Miliar, Ini Alasannya</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 13:14:24 +0700</t>
+          <t>Thu, 03 Sep 2026 20:45:36 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Pelaku sudah diamankan di kantor polisi.</t>
+          <t>Sudaryono menyebut proses pengadaan LED yang tercatat di Inaproc dibatalkan karena alasan pengadaan dinilai tidak tepat dan tidak memiliki pagu anggaran.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283758/pria-nekat-curi-laptop-dan-iphone-di-mal-lalu-disembunyikan-dalam-celana</t>
+          <t>https://www.liputan6.com/news/read/8284208/bgn-batalkan-pengadaan-led-rp535-miliar-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -2344,23 +2337,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Prabowo Bertemu Putin di Vladivostok Bahas Kemitraan Strategis</t>
+          <t>Kehadiran Arya Wedakarna di Miss Equality World 2026 Tuai Sorotan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 12:33:02 +0700</t>
+          <t>Thu, 03 Sep 2026 20:24:47 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Presiden RI Prabowo Subianto menghadiri jamuan santap siang bersama Presiden Rusia Vladimir Putin di Vladivostok, Kamis waktu setempat. Pertemuan tersebut membahas hubungan Indonesia dan Rusia serta agenda Eastern Economic Forum (EEF) ke-11.
-Prabowo menyoroti hubungan kedua negara yang telah berlan</t>
+          <t>Badan Kehormatan DPD akan memanggil I Gusti Ngurah Arya Wedakarna, soal kehadirannya di ajang Miss Equality World 2026 di Bangkok, Thailand.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/photo/read/8283724/prabowo-bertemu-putin-di-vladivostok-bahas-kemitraan-strategis</t>
+          <t>https://www.liputan6.com/news/read/8284199/kehadiran-arya-wedakarna-di-miss-equality-world-2026-tuai-sorotan</t>
         </is>
       </c>
     </row>
@@ -2372,22 +2364,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Momen Prabowo Makan Siang Bareng Putin di Vladivoatok Rusia</t>
+          <t>Wamendagri Ingatkan Kepala Daerah Tak Cukup Hanya Jadi Administrator</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 12:30:57 +0700</t>
+          <t>Thu, 03 Sep 2026 20:15:23 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Prabowo mengaku senang dapat kembali bertemu dengan Putin dan mendapatkan sambutan yang hangat.</t>
+          <t>Wamendagri Akhmad Wiyagus meminta kepala daerah memiliki orientasi strategis, mampu mengantisipasi perubahan, dan berani menghadirkan kebijakan yang berdampak bagi masyarakat.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283723/momen-prabowo-makan-siang-bareng-putin-di-vladivoatok-rusia</t>
+          <t>https://www.liputan6.com/news/read/8284197/wamendagri-ingatkan-kepala-daerah-tak-cukup-hanya-jadi-administrator</t>
         </is>
       </c>
     </row>
@@ -2399,22 +2391,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pesawat Garuda Pecah Ban, Mendarat Darurat di Bandara Sultan Hasanuddin</t>
+          <t>BGN Segera Tempati Kantor Telkom di Graha Merah Putih</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 12:30:29 +0700</t>
+          <t>Thu, 03 Sep 2026 19:53:31 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pesawat jenis Boeing 737-800 itu diketahui mengalami masalah pada ban saat menjalani penerbangan menuju Makassar.</t>
+          <t>BGN tengah berkoordinasi dengan Danantara untuk memindahkan kantor dari gedung yang saat ini berstatus sewa ke Graha Merah Putih.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283720/pesawat-garuda-pecah-ban-mendarat-darurat-di-bandara-sultan-hasanuddin</t>
+          <t>https://www.liputan6.com/news/read/8284182/bgn-segera-tempati-kantor-telkom-di-graha-merah-putih</t>
         </is>
       </c>
     </row>
@@ -2426,22 +2418,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Febrie Adriansyah Ingin Sidang Perkara Segera Digelar</t>
+          <t>Siswi di Matraman yang Hilang Usai Kencan Akhirnya Ditemukan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 12:23:00 +0700</t>
+          <t>Thu, 03 Sep 2026 19:43:02 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kuasa hukumnya Febrie Adriansyah mengatakan, kliennya siap disidang usai permohonan praperadilan ditolak.</t>
+          <t>Siswi SMA berinisial F, yang sebelumnya dilaporkan hilang bersama seorang pria dari aplikasi kencan akhirnya ditemukan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283711/febrie-adriansyah-ingin-sidang-perkara-segera-digelar</t>
+          <t>https://www.liputan6.com/news/read/8284172/siswi-di-matraman-yang-hilang-usai-kencan-akhirnya-ditemukan</t>
         </is>
       </c>
     </row>
@@ -2453,22 +2445,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Bogor Diguncang Gempa</t>
+          <t>Sidang Kuota Haji, Eks Kemenag Akui Ada Tim Cari Alasan Pembagian 50:50</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 11:55:08 +0700</t>
+          <t>Thu, 03 Sep 2026 19:23:15 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gempa pertama terjadi pada pukul 11.23 WIB dengan magnitudo 2,0.</t>
+          <t>Sidang kasus dugaan korupsi kuota haji mengungkap pembentukan tim di Kemenag untuk mencari alasan pembenar pembagian kuota tambahan 2024 secara 50:50.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283683/bogor-diguncang-gempa</t>
+          <t>https://www.liputan6.com/news/read/8284148/sidang-kuota-haji-eks-kemenag-akui-ada-tim-cari-alasan-pembagian-5050</t>
         </is>
       </c>
     </row>
@@ -2480,22 +2472,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kepergok Curi Motor, Maling Panik Nyemplung ke Kali</t>
+          <t>Bareskrim Ungkap Jaringan Judi Online di Balik Spam Komentar Medsos</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 11:37:18 +0700</t>
+          <t>Thu, 03 Sep 2026 19:10:00 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pelaku dipergoki warga saat hendak mencuri sepeda motor di kawasan Jalan Boulevard Raya, Kelapa Gading Timur</t>
+          <t>Bareskrim Polri mengungkap jaringan judi online yang menyebarkan promosi melalui spam komentar di media sosial dengan omzet ditaksir mencapai Rp7,5 miliar per bulan.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283667/kepergok-curi-motor-maling-panik-nyemplung-ke-kali</t>
+          <t>https://www.liputan6.com/news/read/8284134/bareskrim-ungkap-jaringan-judi-online-di-balik-spam-komentar-medsos</t>
         </is>
       </c>
     </row>
@@ -2507,22 +2499,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Penampakan Eks Jampidsus Febrie Tiba di Kejagung untuk Diperiksa TPPU</t>
+          <t>Infografis: Tips Mencegah Kebakaran Saat Musim Kemarau</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 11:36:00 +0700</t>
+          <t>Thu, 03 Sep 2026 19:05:38 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Febrie Adriansyah, eks Jampidsus, tiba dengan pengawalan ketat.</t>
+          <t>Warga diminta mewaspadai kebakaran akibat api terbuka dan listrik.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283665/penampakan-eks-jampidsus-febrie-tiba-di-kejagung-untuk-diperiksa-tppu</t>
+          <t>https://www.liputan6.com/news/read/8284150/infografis-tips-mencegah-kebakaran-saat-musim-kemarau</t>
         </is>
       </c>
     </row>
@@ -2534,22 +2526,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jamin Tak Naik, DPRD Ungkap Awal Polemik Tarif Parkir Rp 60 Ribu per Jam</t>
+          <t>Prabowo Undang Dunia Usaha Rusia: Datang ke Indonesia, Bekerja Bersama Kami</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 03 Sep 2026 11:32:43 +0700</t>
+          <t>Thu, 03 Sep 2026 19:22:46 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Dishub DKI Jakarta juga minta maaf soal tarif parkir Rp 60 ribu jadi polemik.</t>
+          <t>Prabowo menegaskan Indonesia membuka pintu bagi kerja sama ekonomi yang lebih luas dengan Rusia.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8283654/jamin-tak-naik-dprd-ungkap-awal-polemik-tarif-parkir-rp-60-ribu-per-jam</t>
+          <t>https://www.liputan6.com/news/read/8284160/prabowo-undang-dunia-usaha-rusia-datang-ke-indonesia-bekerja-bersama-kami</t>
         </is>
       </c>
     </row>

</xml_diff>